<commit_message>
chore(stats): daily snapshot 2026-04-22
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="README" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -639,7 +639,55 @@
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="19">
-      <c r="A3" s="22" t="n"/>
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>47</v>
+      </c>
+      <c r="C3" t="n">
+        <v>46</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16660</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16456</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="H3" t="n">
+        <v>97</v>
+      </c>
+      <c r="I3" t="n">
+        <v>52</v>
+      </c>
+      <c r="J3" t="n">
+        <v>640</v>
+      </c>
+      <c r="K3" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" t="n">
+        <v>40</v>
+      </c>
+      <c r="N3" t="n">
+        <v>55</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-21.csv</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-04-23
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -644,53 +644,101 @@
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>47</v>
-      </c>
-      <c r="C3" t="n">
-        <v>46</v>
-      </c>
-      <c r="D3" t="n">
-        <v>16660</v>
-      </c>
-      <c r="E3" t="n">
-        <v>16456</v>
-      </c>
-      <c r="F3" t="n">
-        <v>8.960000000000001</v>
-      </c>
-      <c r="G3" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="H3" t="n">
-        <v>97</v>
-      </c>
-      <c r="I3" t="n">
-        <v>52</v>
-      </c>
-      <c r="J3" t="n">
-        <v>640</v>
-      </c>
-      <c r="K3" t="n">
-        <v>8.119999999999999</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="B3" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="C3" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <v>10908</v>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>106459</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="G3" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="H3" s="18" t="n">
+        <v>82</v>
+      </c>
+      <c r="I3" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="J3" s="18" t="n">
+        <v>522</v>
+      </c>
+      <c r="K3" s="18" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="L3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="M3" t="n">
-        <v>40</v>
-      </c>
-      <c r="N3" t="n">
+      <c r="M3" s="18" t="n">
+        <v>38</v>
+      </c>
+      <c r="N3" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" s="18" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-22.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="19">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>55</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>gsc=gsc_queries_2026-04-21.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="19">
-      <c r="A4" s="22" t="n"/>
+      <c r="C4" t="n">
+        <v>55</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10413</v>
+      </c>
+      <c r="E4" t="n">
+        <v>103865</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9.48</v>
+      </c>
+      <c r="G4" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>83</v>
+      </c>
+      <c r="I4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" t="n">
+        <v>541</v>
+      </c>
+      <c r="K4" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>39</v>
+      </c>
+      <c r="N4" t="n">
+        <v>51</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-23.csv</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="19">
       <c r="A5" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-04-24
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -695,53 +695,101 @@
           <t>2026-04-23</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="18" t="n">
         <v>10413</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="18" t="n">
         <v>103865</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="18" t="n">
         <v>9.48</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="18" t="n">
         <v>83</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="18" t="n">
         <v>541</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="18" t="n">
         <v>9.24</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="18" t="n">
         <v>51</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-04-23.csv</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="19">
-      <c r="A5" s="22" t="n"/>
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10137</v>
+      </c>
+      <c r="E5" t="n">
+        <v>102355</v>
+      </c>
+      <c r="F5" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>85</v>
+      </c>
+      <c r="I5" t="n">
+        <v>51</v>
+      </c>
+      <c r="J5" t="n">
+        <v>554</v>
+      </c>
+      <c r="K5" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>41</v>
+      </c>
+      <c r="N5" t="n">
+        <v>52</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-24.csv</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="19">
       <c r="A6" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-04-25
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -746,53 +746,101 @@
           <t>2026-04-24</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="18" t="n">
         <v>10137</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="18" t="n">
         <v>102355</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="18" t="n">
         <v>9.359999999999999</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="18" t="n">
         <v>51</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="18" t="n">
         <v>554</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="18" t="n">
         <v>9.210000000000001</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="18" t="n">
         <v>52</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-04-24.csv</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="19">
-      <c r="A6" s="22" t="n"/>
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>55</v>
+      </c>
+      <c r="C6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9385</v>
+      </c>
+      <c r="E6" t="n">
+        <v>95462</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="G6" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>90</v>
+      </c>
+      <c r="I6" t="n">
+        <v>56</v>
+      </c>
+      <c r="J6" t="n">
+        <v>578</v>
+      </c>
+      <c r="K6" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="n">
+        <v>41</v>
+      </c>
+      <c r="N6" t="n">
+        <v>54</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-25.csv</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="19">
       <c r="A7" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-04-26
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -797,53 +797,101 @@
           <t>2026-04-25</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="18" t="n">
         <v>9385</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="18" t="n">
         <v>95462</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="18" t="n">
         <v>9.25</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="18" t="n">
         <v>56</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="18" t="n">
         <v>578</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="18" t="n">
         <v>9.69</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="18" t="n">
         <v>54</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-04-25.csv</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="19">
-      <c r="A7" s="22" t="n"/>
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>55</v>
+      </c>
+      <c r="C7" t="n">
+        <v>55</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9054</v>
+      </c>
+      <c r="E7" t="n">
+        <v>92089</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="G7" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>90</v>
+      </c>
+      <c r="I7" t="n">
+        <v>55</v>
+      </c>
+      <c r="J7" t="n">
+        <v>572</v>
+      </c>
+      <c r="K7" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" t="n">
+        <v>41</v>
+      </c>
+      <c r="N7" t="n">
+        <v>54</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-26.csv</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="19">
       <c r="A8" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-04-29
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -848,53 +848,101 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="18" t="n">
         <v>9054</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="18" t="n">
         <v>92089</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="18" t="n">
         <v>9.220000000000001</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="18" t="n">
         <v>47.2</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="18" t="n">
         <v>572</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="18" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="18" t="n">
         <v>54</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-04-26.csv</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="19">
-      <c r="A8" s="22" t="n"/>
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>55</v>
+      </c>
+      <c r="C8" t="n">
+        <v>55</v>
+      </c>
+      <c r="D8" t="n">
+        <v>7869</v>
+      </c>
+      <c r="E8" t="n">
+        <v>82087</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="H8" t="n">
+        <v>107</v>
+      </c>
+      <c r="I8" t="n">
+        <v>57</v>
+      </c>
+      <c r="J8" t="n">
+        <v>716</v>
+      </c>
+      <c r="K8" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" t="n">
+        <v>50</v>
+      </c>
+      <c r="N8" t="n">
+        <v>69</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-29.csv</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="19">
       <c r="A9" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-04-30
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -899,53 +899,101 @@
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="18" t="n">
         <v>7869</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="18" t="n">
         <v>82087</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="18" t="n">
         <v>8.9</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="18" t="n">
         <v>47.9</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="18" t="n">
         <v>107</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="18" t="n">
         <v>57</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="18" t="n">
         <v>716</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="18" t="n">
         <v>7.96</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-04-29.csv</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="19">
-      <c r="A9" s="22" t="n"/>
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>55</v>
+      </c>
+      <c r="C9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6918</v>
+      </c>
+      <c r="E9" t="n">
+        <v>73637</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.630000000000001</v>
+      </c>
+      <c r="G9" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>108</v>
+      </c>
+      <c r="I9" t="n">
+        <v>57</v>
+      </c>
+      <c r="J9" t="n">
+        <v>741</v>
+      </c>
+      <c r="K9" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>50</v>
+      </c>
+      <c r="N9" t="n">
+        <v>70</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-04-30.csv</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="19">
       <c r="A10" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-01
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -950,53 +950,101 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="18" t="n">
         <v>6918</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="18" t="n">
         <v>73637</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="18" t="n">
         <v>8.630000000000001</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="18" t="n">
         <v>108</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="18" t="n">
         <v>57</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="18" t="n">
         <v>741</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="18" t="n">
         <v>7.69</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-04-30.csv</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="19">
-      <c r="A10" s="22" t="n"/>
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>55</v>
+      </c>
+      <c r="C10" t="n">
+        <v>55</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6384</v>
+      </c>
+      <c r="E10" t="n">
+        <v>69130</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="G10" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>108</v>
+      </c>
+      <c r="I10" t="n">
+        <v>61</v>
+      </c>
+      <c r="J10" t="n">
+        <v>775</v>
+      </c>
+      <c r="K10" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>50</v>
+      </c>
+      <c r="N10" t="n">
+        <v>70</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-01.csv</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="19">
       <c r="A11" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-02
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1001,53 +1001,101 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="18" t="n">
         <v>6384</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="18" t="n">
         <v>69130</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="18" t="n">
         <v>8.42</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="18" t="n">
         <v>48.3</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="18" t="n">
         <v>108</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="18" t="n">
         <v>61</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="18" t="n">
         <v>775</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="18" t="n">
         <v>7.87</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-01.csv</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="19">
-      <c r="A11" s="22" t="n"/>
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>55</v>
+      </c>
+      <c r="C11" t="n">
+        <v>55</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5967</v>
+      </c>
+      <c r="E11" t="n">
+        <v>65304</v>
+      </c>
+      <c r="F11" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="G11" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>112</v>
+      </c>
+      <c r="I11" t="n">
+        <v>65</v>
+      </c>
+      <c r="J11" t="n">
+        <v>814</v>
+      </c>
+      <c r="K11" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>52</v>
+      </c>
+      <c r="N11" t="n">
+        <v>73</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-02.csv</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="19">
       <c r="A12" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-03
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1052,53 +1052,101 @@
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="18" t="n">
         <v>5967</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="18" t="n">
         <v>65304</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="18" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="18" t="n">
         <v>48.2</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="18" t="n">
         <v>112</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="18" t="n">
         <v>65</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="18" t="n">
         <v>814</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="18" t="n">
         <v>7.99</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="18" t="n">
         <v>52</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-02.csv</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="19">
-      <c r="A12" s="22" t="n"/>
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>55</v>
+      </c>
+      <c r="C12" t="n">
+        <v>55</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5716</v>
+      </c>
+      <c r="E12" t="n">
+        <v>62559</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="G12" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>130</v>
+      </c>
+      <c r="I12" t="n">
+        <v>70</v>
+      </c>
+      <c r="J12" t="n">
+        <v>879</v>
+      </c>
+      <c r="K12" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="L12" t="n">
+        <v>5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>56</v>
+      </c>
+      <c r="N12" t="n">
+        <v>75</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-03.csv</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="19">
       <c r="A13" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-04
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1103,53 +1103,101 @@
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="18" t="n">
         <v>5716</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="18" t="n">
         <v>62559</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="18" t="n">
         <v>8.24</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" s="18" t="n">
         <v>879</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="18" t="n">
         <v>7.96</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="18" t="n">
         <v>56</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-03.csv</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="19">
-      <c r="A13" s="22" t="n"/>
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>55</v>
+      </c>
+      <c r="C13" t="n">
+        <v>55</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5533</v>
+      </c>
+      <c r="E13" t="n">
+        <v>61307</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="G13" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="H13" t="n">
+        <v>144</v>
+      </c>
+      <c r="I13" t="n">
+        <v>73</v>
+      </c>
+      <c r="J13" t="n">
+        <v>941</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="L13" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>57</v>
+      </c>
+      <c r="N13" t="n">
+        <v>78</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-04.csv</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="19">
       <c r="A14" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-05
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1154,53 +1154,101 @@
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="18" t="n">
         <v>5533</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="18" t="n">
         <v>61307</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="18" t="n">
         <v>8.109999999999999</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="18" t="n">
         <v>48.6</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="18" t="n">
         <v>144</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="18" t="n">
         <v>941</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="18" t="n">
         <v>7.76</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="18" t="n">
         <v>57</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-04.csv</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="19">
-      <c r="A14" s="22" t="n"/>
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>55</v>
+      </c>
+      <c r="C14" t="n">
+        <v>55</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5334</v>
+      </c>
+      <c r="E14" t="n">
+        <v>59214</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="G14" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>146</v>
+      </c>
+      <c r="I14" t="n">
+        <v>71</v>
+      </c>
+      <c r="J14" t="n">
+        <v>941</v>
+      </c>
+      <c r="K14" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="L14" t="n">
+        <v>4</v>
+      </c>
+      <c r="M14" t="n">
+        <v>59</v>
+      </c>
+      <c r="N14" t="n">
+        <v>80</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-05.csv</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="19">
       <c r="A15" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-06
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1205,53 +1205,101 @@
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="18" t="n">
         <v>5334</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="18" t="n">
         <v>59214</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="18" t="n">
         <v>8.06</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="18" t="n">
         <v>47.6</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="18" t="n">
         <v>146</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="18" t="n">
         <v>71</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" s="18" t="n">
         <v>941</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="18" t="n">
         <v>7.55</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="18" t="n">
         <v>59</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N14" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-05.csv</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="19">
-      <c r="A15" s="22" t="n"/>
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>55</v>
+      </c>
+      <c r="C15" t="n">
+        <v>55</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5204</v>
+      </c>
+      <c r="E15" t="n">
+        <v>58208</v>
+      </c>
+      <c r="F15" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="G15" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="H15" t="n">
+        <v>148</v>
+      </c>
+      <c r="I15" t="n">
+        <v>71</v>
+      </c>
+      <c r="J15" t="n">
+        <v>957</v>
+      </c>
+      <c r="K15" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="L15" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" t="n">
+        <v>60</v>
+      </c>
+      <c r="N15" t="n">
+        <v>83</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-06.csv</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="19">
       <c r="A16" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-07
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1256,53 +1256,101 @@
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="18" t="n">
         <v>5204</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="18" t="n">
         <v>58208</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="18" t="n">
         <v>7.98</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="18" t="n">
         <v>47.9</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="18" t="n">
         <v>148</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="18" t="n">
         <v>71</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="18" t="n">
         <v>957</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" s="18" t="n">
         <v>7.42</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N15" s="18" t="n">
         <v>83</v>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-06.csv</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="19">
-      <c r="A16" s="22" t="n"/>
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>55</v>
+      </c>
+      <c r="C16" t="n">
+        <v>55</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5084</v>
+      </c>
+      <c r="E16" t="n">
+        <v>57271</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G16" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>147</v>
+      </c>
+      <c r="I16" t="n">
+        <v>68</v>
+      </c>
+      <c r="J16" t="n">
+        <v>969</v>
+      </c>
+      <c r="K16" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="L16" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>58</v>
+      </c>
+      <c r="N16" t="n">
+        <v>81</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-07.csv</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="19">
       <c r="A17" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-08
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1307,53 +1307,101 @@
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="18" t="n">
         <v>5084</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="18" t="n">
         <v>57271</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="18" t="n">
         <v>7.9</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="18" t="n">
         <v>48.3</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="18" t="n">
         <v>147</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="18" t="n">
         <v>68</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="18" t="n">
         <v>969</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="18" t="n">
         <v>7.02</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="18" t="n">
         <v>58</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16" s="18" t="n">
         <v>81</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-07.csv</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="19">
-      <c r="A17" s="22" t="n"/>
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>55</v>
+      </c>
+      <c r="C17" t="n">
+        <v>55</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5041</v>
+      </c>
+      <c r="E17" t="n">
+        <v>57282</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="G17" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>150</v>
+      </c>
+      <c r="I17" t="n">
+        <v>68</v>
+      </c>
+      <c r="J17" t="n">
+        <v>975</v>
+      </c>
+      <c r="K17" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="L17" t="n">
+        <v>5</v>
+      </c>
+      <c r="M17" t="n">
+        <v>60</v>
+      </c>
+      <c r="N17" t="n">
+        <v>82</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-08.csv</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="19">
       <c r="A18" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-09
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1358,53 +1358,101 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="18" t="n">
         <v>5041</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="18" t="n">
         <v>57282</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="18" t="n">
         <v>7.82</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="18" t="n">
         <v>49.3</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="18" t="n">
         <v>68</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="18" t="n">
         <v>975</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="18" t="n">
         <v>6.97</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L17" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-08.csv</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="19">
-      <c r="A18" s="22" t="n"/>
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>55</v>
+      </c>
+      <c r="C18" t="n">
+        <v>55</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4978</v>
+      </c>
+      <c r="E18" t="n">
+        <v>57191</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="G18" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H18" t="n">
+        <v>152</v>
+      </c>
+      <c r="I18" t="n">
+        <v>67</v>
+      </c>
+      <c r="J18" t="n">
+        <v>973</v>
+      </c>
+      <c r="K18" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="L18" t="n">
+        <v>5</v>
+      </c>
+      <c r="M18" t="n">
+        <v>59</v>
+      </c>
+      <c r="N18" t="n">
+        <v>84</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-09.csv</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="19">
       <c r="A19" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-10
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1409,53 +1409,101 @@
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="18" t="n">
         <v>4978</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="18" t="n">
         <v>57191</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="18" t="n">
         <v>7.72</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="18" t="n">
         <v>48.9</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H18" s="18" t="n">
         <v>152</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" s="18" t="n">
         <v>67</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J18" s="18" t="n">
         <v>973</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" s="18" t="n">
         <v>6.89</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L18" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" s="18" t="n">
         <v>59</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N18" s="18" t="n">
         <v>84</v>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O18" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-09.csv</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="19">
-      <c r="A19" s="22" t="n"/>
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>55</v>
+      </c>
+      <c r="C19" t="n">
+        <v>55</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4948</v>
+      </c>
+      <c r="E19" t="n">
+        <v>57583</v>
+      </c>
+      <c r="F19" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="G19" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>157</v>
+      </c>
+      <c r="I19" t="n">
+        <v>71</v>
+      </c>
+      <c r="J19" t="n">
+        <v>982</v>
+      </c>
+      <c r="K19" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="L19" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" t="n">
+        <v>62</v>
+      </c>
+      <c r="N19" t="n">
+        <v>87</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-10.csv</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="19">
       <c r="A20" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-11
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1460,53 +1460,101 @@
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="18" t="n">
         <v>4948</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="18" t="n">
         <v>57583</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="18" t="n">
         <v>7.62</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="18" t="n">
         <v>49.5</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="18" t="n">
         <v>157</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="18" t="n">
         <v>71</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="18" t="n">
         <v>982</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="18" t="n">
         <v>7.23</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L19" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" s="18" t="n">
         <v>62</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" s="18" t="n">
         <v>87</v>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O19" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-10.csv</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="19">
-      <c r="A20" s="22" t="n"/>
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>55</v>
+      </c>
+      <c r="C20" t="n">
+        <v>55</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4919</v>
+      </c>
+      <c r="E20" t="n">
+        <v>57980</v>
+      </c>
+      <c r="F20" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="G20" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>161</v>
+      </c>
+      <c r="I20" t="n">
+        <v>70</v>
+      </c>
+      <c r="J20" t="n">
+        <v>979</v>
+      </c>
+      <c r="K20" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="L20" t="n">
+        <v>6</v>
+      </c>
+      <c r="M20" t="n">
+        <v>63</v>
+      </c>
+      <c r="N20" t="n">
+        <v>90</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-11.csv</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="19">
       <c r="A21" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-12
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1511,53 +1511,101 @@
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="18" t="n">
         <v>4919</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="18" t="n">
         <v>57980</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="18" t="n">
         <v>7.52</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="18" t="n">
         <v>50.1</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" s="18" t="n">
         <v>161</v>
       </c>
-      <c r="I20" t="n">
+      <c r="I20" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="J20" t="n">
+      <c r="J20" s="18" t="n">
         <v>979</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" s="18" t="n">
         <v>7.15</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L20" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" s="18" t="n">
         <v>63</v>
       </c>
-      <c r="N20" t="n">
+      <c r="N20" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O20" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-11.csv</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="19">
-      <c r="A21" s="22" t="n"/>
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>55</v>
+      </c>
+      <c r="C21" t="n">
+        <v>55</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4800</v>
+      </c>
+      <c r="E21" t="n">
+        <v>56708</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="G21" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="H21" t="n">
+        <v>161</v>
+      </c>
+      <c r="I21" t="n">
+        <v>64</v>
+      </c>
+      <c r="J21" t="n">
+        <v>975</v>
+      </c>
+      <c r="K21" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="L21" t="n">
+        <v>6</v>
+      </c>
+      <c r="M21" t="n">
+        <v>64</v>
+      </c>
+      <c r="N21" t="n">
+        <v>91</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-12.csv</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="19">
       <c r="A22" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-21
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1562,53 +1562,101 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="18" t="n">
         <v>4800</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="18" t="n">
         <v>56708</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="18" t="n">
         <v>7.47</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" s="18" t="n">
         <v>49.9</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="18" t="n">
         <v>161</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" s="18" t="n">
         <v>64</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" s="18" t="n">
         <v>975</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" s="18" t="n">
         <v>6.56</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L21" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="M21" t="n">
+      <c r="M21" s="18" t="n">
         <v>64</v>
       </c>
-      <c r="N21" t="n">
+      <c r="N21" s="18" t="n">
         <v>91</v>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O21" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-12.csv</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="19">
-      <c r="A22" s="22" t="n"/>
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>55</v>
+      </c>
+      <c r="C22" t="n">
+        <v>55</v>
+      </c>
+      <c r="D22" t="n">
+        <v>4586</v>
+      </c>
+      <c r="E22" t="n">
+        <v>54942</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="G22" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="H22" t="n">
+        <v>161</v>
+      </c>
+      <c r="I22" t="n">
+        <v>69</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1067</v>
+      </c>
+      <c r="K22" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="L22" t="n">
+        <v>7</v>
+      </c>
+      <c r="M22" t="n">
+        <v>69</v>
+      </c>
+      <c r="N22" t="n">
+        <v>96</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-21.csv</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="19">
       <c r="A23" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-26
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1613,53 +1613,101 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="18" t="n">
         <v>4586</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="18" t="n">
         <v>54942</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="18" t="n">
         <v>7.33</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="18" t="n">
         <v>49.7</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" s="18" t="n">
         <v>161</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="J22" t="n">
+      <c r="J22" s="18" t="n">
         <v>1067</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" s="18" t="n">
         <v>6.47</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L22" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="M22" t="n">
+      <c r="M22" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="N22" t="n">
+      <c r="N22" s="18" t="n">
         <v>96</v>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O22" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-21.csv</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="19">
-      <c r="A23" s="22" t="n"/>
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>55</v>
+      </c>
+      <c r="C23" t="n">
+        <v>55</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4581</v>
+      </c>
+      <c r="E23" t="n">
+        <v>51630</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7.79</v>
+      </c>
+      <c r="G23" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>156</v>
+      </c>
+      <c r="I23" t="n">
+        <v>69</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1069</v>
+      </c>
+      <c r="K23" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="L23" t="n">
+        <v>8</v>
+      </c>
+      <c r="M23" t="n">
+        <v>71</v>
+      </c>
+      <c r="N23" t="n">
+        <v>97</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-26.csv</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="19">
       <c r="A24" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-28
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1664,53 +1664,101 @@
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="18" t="n">
         <v>4581</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="18" t="n">
         <v>51630</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="18" t="n">
         <v>7.79</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="18" t="n">
         <v>48.2</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H23" s="18" t="n">
         <v>156</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" s="18" t="n">
         <v>1069</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" s="18" t="n">
         <v>6.45</v>
       </c>
-      <c r="L23" t="n">
+      <c r="L23" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="M23" t="n">
+      <c r="M23" s="18" t="n">
         <v>71</v>
       </c>
-      <c r="N23" t="n">
+      <c r="N23" s="18" t="n">
         <v>97</v>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O23" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-26.csv</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="19">
-      <c r="A24" s="22" t="n"/>
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>55</v>
+      </c>
+      <c r="C24" t="n">
+        <v>55</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4418</v>
+      </c>
+      <c r="E24" t="n">
+        <v>48894</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="G24" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="H24" t="n">
+        <v>161</v>
+      </c>
+      <c r="I24" t="n">
+        <v>68</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1105</v>
+      </c>
+      <c r="K24" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="L24" t="n">
+        <v>8</v>
+      </c>
+      <c r="M24" t="n">
+        <v>73</v>
+      </c>
+      <c r="N24" t="n">
+        <v>104</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-28.csv</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="19">
       <c r="A25" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily snapshot 2026-05-29
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1715,53 +1715,101 @@
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="18" t="n">
         <v>4418</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="18" t="n">
         <v>48894</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="18" t="n">
         <v>7.89</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" s="18" t="n">
         <v>46.9</v>
       </c>
-      <c r="H24" t="n">
+      <c r="H24" s="18" t="n">
         <v>161</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I24" s="18" t="n">
         <v>68</v>
       </c>
-      <c r="J24" t="n">
+      <c r="J24" s="18" t="n">
         <v>1105</v>
       </c>
-      <c r="K24" t="n">
+      <c r="K24" s="18" t="n">
         <v>6.15</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L24" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="M24" t="n">
+      <c r="M24" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="N24" t="n">
+      <c r="N24" s="18" t="n">
         <v>104</v>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O24" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-28.csv</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="19">
-      <c r="A25" s="22" t="n"/>
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>55</v>
+      </c>
+      <c r="C25" t="n">
+        <v>53</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4347</v>
+      </c>
+      <c r="E25" t="n">
+        <v>47843</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="G25" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="H25" t="n">
+        <v>163</v>
+      </c>
+      <c r="I25" t="n">
+        <v>66</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1107</v>
+      </c>
+      <c r="K25" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="L25" t="n">
+        <v>8</v>
+      </c>
+      <c r="M25" t="n">
+        <v>75</v>
+      </c>
+      <c r="N25" t="n">
+        <v>109</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-29.csv</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="19">
       <c r="A26" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-17
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="README" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1766,53 +1766,101 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="18" t="n">
         <v>53</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" s="18" t="n">
         <v>4347</v>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="18" t="n">
         <v>47843</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="18" t="n">
         <v>7.91</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="18" t="n">
         <v>46.6</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" s="18" t="n">
         <v>163</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" s="18" t="n">
         <v>66</v>
       </c>
-      <c r="J25" t="n">
+      <c r="J25" s="18" t="n">
         <v>1107</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" s="18" t="n">
         <v>5.96</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L25" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="M25" t="n">
+      <c r="M25" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="N25" t="n">
+      <c r="N25" s="18" t="n">
         <v>109</v>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="O25" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-05-29.csv</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="19">
-      <c r="A26" s="22" t="n"/>
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>55</v>
+      </c>
+      <c r="C26" t="n">
+        <v>53</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4347</v>
+      </c>
+      <c r="E26" t="n">
+        <v>47843</v>
+      </c>
+      <c r="F26" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="G26" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>161</v>
+      </c>
+      <c r="I26" t="n">
+        <v>68</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1105</v>
+      </c>
+      <c r="K26" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="L26" t="n">
+        <v>8</v>
+      </c>
+      <c r="M26" t="n">
+        <v>73</v>
+      </c>
+      <c r="N26" t="n">
+        <v>104</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-05-28.csv</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="19">
       <c r="A27" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-18
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1863,7 +1863,55 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="19">
-      <c r="A27" s="22" t="n"/>
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>75</v>
+      </c>
+      <c r="C27" t="n">
+        <v>73</v>
+      </c>
+      <c r="D27" t="n">
+        <v>74875</v>
+      </c>
+      <c r="E27" t="n">
+        <v>547329</v>
+      </c>
+      <c r="F27" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="G27" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>201</v>
+      </c>
+      <c r="I27" t="n">
+        <v>94</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1548</v>
+      </c>
+      <c r="K27" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="L27" t="n">
+        <v>14</v>
+      </c>
+      <c r="M27" t="n">
+        <v>135</v>
+      </c>
+      <c r="N27" t="n">
+        <v>174</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-18.csv</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="19">
       <c r="A28" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-19
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1868,53 +1868,101 @@
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="18" t="n">
         <v>74875</v>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="18" t="n">
         <v>547329</v>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="18" t="n">
         <v>13.58</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" s="18" t="n">
         <v>48.2</v>
       </c>
-      <c r="H27" t="n">
+      <c r="H27" s="18" t="n">
         <v>201</v>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" s="18" t="n">
         <v>94</v>
       </c>
-      <c r="J27" t="n">
+      <c r="J27" s="18" t="n">
         <v>1548</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K27" s="18" t="n">
         <v>6.07</v>
       </c>
-      <c r="L27" t="n">
+      <c r="L27" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="M27" t="n">
+      <c r="M27" s="18" t="n">
         <v>135</v>
       </c>
-      <c r="N27" t="n">
+      <c r="N27" s="18" t="n">
         <v>174</v>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O27" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-18.csv</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="19">
-      <c r="A28" s="22" t="n"/>
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>75</v>
+      </c>
+      <c r="C28" t="n">
+        <v>73</v>
+      </c>
+      <c r="D28" t="n">
+        <v>74986</v>
+      </c>
+      <c r="E28" t="n">
+        <v>548713</v>
+      </c>
+      <c r="F28" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="G28" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="H28" t="n">
+        <v>208</v>
+      </c>
+      <c r="I28" t="n">
+        <v>102</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1615</v>
+      </c>
+      <c r="K28" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="L28" t="n">
+        <v>13</v>
+      </c>
+      <c r="M28" t="n">
+        <v>134</v>
+      </c>
+      <c r="N28" t="n">
+        <v>181</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-19.csv</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="19">
       <c r="A29" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-20
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1919,53 +1919,101 @@
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="18" t="n">
         <v>74986</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="18" t="n">
         <v>548713</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="18" t="n">
         <v>13.56</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" s="18" t="n">
         <v>48.3</v>
       </c>
-      <c r="H28" t="n">
+      <c r="H28" s="18" t="n">
         <v>208</v>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" s="18" t="n">
         <v>102</v>
       </c>
-      <c r="J28" t="n">
+      <c r="J28" s="18" t="n">
         <v>1615</v>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" s="18" t="n">
         <v>6.32</v>
       </c>
-      <c r="L28" t="n">
+      <c r="L28" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="M28" t="n">
+      <c r="M28" s="18" t="n">
         <v>134</v>
       </c>
-      <c r="N28" t="n">
+      <c r="N28" s="18" t="n">
         <v>181</v>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O28" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-19.csv</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="19">
-      <c r="A29" s="22" t="n"/>
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>75</v>
+      </c>
+      <c r="C29" t="n">
+        <v>73</v>
+      </c>
+      <c r="D29" t="n">
+        <v>73596</v>
+      </c>
+      <c r="E29" t="n">
+        <v>546902</v>
+      </c>
+      <c r="F29" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="G29" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>208</v>
+      </c>
+      <c r="I29" t="n">
+        <v>106</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1652</v>
+      </c>
+      <c r="K29" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="L29" t="n">
+        <v>13</v>
+      </c>
+      <c r="M29" t="n">
+        <v>136</v>
+      </c>
+      <c r="N29" t="n">
+        <v>183</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-20.csv</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="19">
       <c r="A30" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-21
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -1970,53 +1970,101 @@
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="18" t="n">
         <v>73596</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="18" t="n">
         <v>546902</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="18" t="n">
         <v>13.35</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" s="18" t="n">
         <v>48.2</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H29" s="18" t="n">
         <v>208</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" s="18" t="n">
         <v>106</v>
       </c>
-      <c r="J29" t="n">
+      <c r="J29" s="18" t="n">
         <v>1652</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K29" s="18" t="n">
         <v>6.42</v>
       </c>
-      <c r="L29" t="n">
+      <c r="L29" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="M29" t="n">
+      <c r="M29" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="N29" t="n">
+      <c r="N29" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O29" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-20.csv</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="19">
-      <c r="A30" s="22" t="n"/>
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>75</v>
+      </c>
+      <c r="C30" t="n">
+        <v>73</v>
+      </c>
+      <c r="D30" t="n">
+        <v>73405</v>
+      </c>
+      <c r="E30" t="n">
+        <v>547958</v>
+      </c>
+      <c r="F30" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="G30" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>209</v>
+      </c>
+      <c r="I30" t="n">
+        <v>107</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1651</v>
+      </c>
+      <c r="K30" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="L30" t="n">
+        <v>13</v>
+      </c>
+      <c r="M30" t="n">
+        <v>137</v>
+      </c>
+      <c r="N30" t="n">
+        <v>181</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-21.csv</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="19">
       <c r="A31" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-22
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2021,53 +2021,101 @@
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="18" t="n">
         <v>73405</v>
       </c>
-      <c r="E30" t="n">
+      <c r="E30" s="18" t="n">
         <v>547958</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" s="18" t="n">
         <v>13.29</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G30" s="18" t="n">
         <v>48.2</v>
       </c>
-      <c r="H30" t="n">
+      <c r="H30" s="18" t="n">
         <v>209</v>
       </c>
-      <c r="I30" t="n">
+      <c r="I30" s="18" t="n">
         <v>107</v>
       </c>
-      <c r="J30" t="n">
+      <c r="J30" s="18" t="n">
         <v>1651</v>
       </c>
-      <c r="K30" t="n">
+      <c r="K30" s="18" t="n">
         <v>6.48</v>
       </c>
-      <c r="L30" t="n">
+      <c r="L30" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="M30" t="n">
+      <c r="M30" s="18" t="n">
         <v>137</v>
       </c>
-      <c r="N30" t="n">
+      <c r="N30" s="18" t="n">
         <v>181</v>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="O30" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-21.csv</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="19">
-      <c r="A31" s="22" t="n"/>
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>75</v>
+      </c>
+      <c r="C31" t="n">
+        <v>73</v>
+      </c>
+      <c r="D31" t="n">
+        <v>71955</v>
+      </c>
+      <c r="E31" t="n">
+        <v>535019</v>
+      </c>
+      <c r="F31" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="G31" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H31" t="n">
+        <v>210</v>
+      </c>
+      <c r="I31" t="n">
+        <v>104</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1696</v>
+      </c>
+      <c r="K31" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="L31" t="n">
+        <v>13</v>
+      </c>
+      <c r="M31" t="n">
+        <v>136</v>
+      </c>
+      <c r="N31" t="n">
+        <v>182</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-22.csv</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="19">
       <c r="A32" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-23
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2072,53 +2072,101 @@
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="18" t="n">
         <v>71955</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="18" t="n">
         <v>535019</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="18" t="n">
         <v>13.35</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H31" t="n">
+      <c r="H31" s="18" t="n">
         <v>210</v>
       </c>
-      <c r="I31" t="n">
+      <c r="I31" s="18" t="n">
         <v>104</v>
       </c>
-      <c r="J31" t="n">
+      <c r="J31" s="18" t="n">
         <v>1696</v>
       </c>
-      <c r="K31" t="n">
+      <c r="K31" s="18" t="n">
         <v>6.13</v>
       </c>
-      <c r="L31" t="n">
+      <c r="L31" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="M31" t="n">
+      <c r="M31" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="N31" t="n">
+      <c r="N31" s="18" t="n">
         <v>182</v>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O31" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-22.csv</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="19">
-      <c r="A32" s="22" t="n"/>
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>76</v>
+      </c>
+      <c r="C32" t="n">
+        <v>73</v>
+      </c>
+      <c r="D32" t="n">
+        <v>71191</v>
+      </c>
+      <c r="E32" t="n">
+        <v>526800</v>
+      </c>
+      <c r="F32" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="G32" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>209</v>
+      </c>
+      <c r="I32" t="n">
+        <v>105</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1699</v>
+      </c>
+      <c r="K32" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="L32" t="n">
+        <v>13</v>
+      </c>
+      <c r="M32" t="n">
+        <v>136</v>
+      </c>
+      <c r="N32" t="n">
+        <v>181</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-23.csv</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="19">
       <c r="A33" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-24
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2123,53 +2123,101 @@
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="18" t="n">
         <v>71191</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="18" t="n">
         <v>526800</v>
       </c>
-      <c r="F32" t="n">
+      <c r="F32" s="18" t="n">
         <v>13.41</v>
       </c>
-      <c r="G32" t="n">
+      <c r="G32" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H32" t="n">
+      <c r="H32" s="18" t="n">
         <v>209</v>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" s="18" t="n">
         <v>105</v>
       </c>
-      <c r="J32" t="n">
+      <c r="J32" s="18" t="n">
         <v>1699</v>
       </c>
-      <c r="K32" t="n">
+      <c r="K32" s="18" t="n">
         <v>6.18</v>
       </c>
-      <c r="L32" t="n">
+      <c r="L32" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="M32" t="n">
+      <c r="M32" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="N32" t="n">
+      <c r="N32" s="18" t="n">
         <v>181</v>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="O32" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-23.csv</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="19">
-      <c r="A33" s="22" t="n"/>
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>76</v>
+      </c>
+      <c r="C33" t="n">
+        <v>73</v>
+      </c>
+      <c r="D33" t="n">
+        <v>67112</v>
+      </c>
+      <c r="E33" t="n">
+        <v>490825</v>
+      </c>
+      <c r="F33" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="G33" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H33" t="n">
+        <v>209</v>
+      </c>
+      <c r="I33" t="n">
+        <v>106</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1713</v>
+      </c>
+      <c r="K33" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="L33" t="n">
+        <v>13</v>
+      </c>
+      <c r="M33" t="n">
+        <v>136</v>
+      </c>
+      <c r="N33" t="n">
+        <v>180</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-24.csv</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="19">
       <c r="A34" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-25
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2174,53 +2174,101 @@
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="18" t="n">
         <v>67112</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="18" t="n">
         <v>490825</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="18" t="n">
         <v>13.56</v>
       </c>
-      <c r="G33" t="n">
+      <c r="G33" s="18" t="n">
         <v>47.6</v>
       </c>
-      <c r="H33" t="n">
+      <c r="H33" s="18" t="n">
         <v>209</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" s="18" t="n">
         <v>106</v>
       </c>
-      <c r="J33" t="n">
+      <c r="J33" s="18" t="n">
         <v>1713</v>
       </c>
-      <c r="K33" t="n">
+      <c r="K33" s="18" t="n">
         <v>6.19</v>
       </c>
-      <c r="L33" t="n">
+      <c r="L33" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="M33" t="n">
+      <c r="M33" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="N33" t="n">
+      <c r="N33" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="O33" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-24.csv</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="19">
-      <c r="A34" s="22" t="n"/>
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>76</v>
+      </c>
+      <c r="C34" t="n">
+        <v>74</v>
+      </c>
+      <c r="D34" t="n">
+        <v>65460</v>
+      </c>
+      <c r="E34" t="n">
+        <v>473798</v>
+      </c>
+      <c r="F34" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G34" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>211</v>
+      </c>
+      <c r="I34" t="n">
+        <v>112</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1739</v>
+      </c>
+      <c r="K34" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="L34" t="n">
+        <v>14</v>
+      </c>
+      <c r="M34" t="n">
+        <v>136</v>
+      </c>
+      <c r="N34" t="n">
+        <v>183</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-25.csv</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="19">
       <c r="A35" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-26
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2225,53 +2225,101 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" s="18" t="n">
         <v>65460</v>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="18" t="n">
         <v>473798</v>
       </c>
-      <c r="F34" t="n">
+      <c r="F34" s="18" t="n">
         <v>13.7</v>
       </c>
-      <c r="G34" t="n">
+      <c r="G34" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H34" t="n">
+      <c r="H34" s="18" t="n">
         <v>211</v>
       </c>
-      <c r="I34" t="n">
+      <c r="I34" s="18" t="n">
         <v>112</v>
       </c>
-      <c r="J34" t="n">
+      <c r="J34" s="18" t="n">
         <v>1739</v>
       </c>
-      <c r="K34" t="n">
+      <c r="K34" s="18" t="n">
         <v>6.44</v>
       </c>
-      <c r="L34" t="n">
+      <c r="L34" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="M34" t="n">
+      <c r="M34" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="N34" t="n">
+      <c r="N34" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="O34" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-25.csv</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="19">
-      <c r="A35" s="22" t="n"/>
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>76</v>
+      </c>
+      <c r="C35" t="n">
+        <v>74</v>
+      </c>
+      <c r="D35" t="n">
+        <v>64790</v>
+      </c>
+      <c r="E35" t="n">
+        <v>467665</v>
+      </c>
+      <c r="F35" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="G35" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>215</v>
+      </c>
+      <c r="I35" t="n">
+        <v>112</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1769</v>
+      </c>
+      <c r="K35" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="L35" t="n">
+        <v>17</v>
+      </c>
+      <c r="M35" t="n">
+        <v>140</v>
+      </c>
+      <c r="N35" t="n">
+        <v>186</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-26.csv</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="19">
       <c r="A36" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-27
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2276,53 +2276,101 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="18" t="n">
         <v>64790</v>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="18" t="n">
         <v>467665</v>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" s="18" t="n">
         <v>13.73</v>
       </c>
-      <c r="G35" t="n">
+      <c r="G35" s="18" t="n">
         <v>47.4</v>
       </c>
-      <c r="H35" t="n">
+      <c r="H35" s="18" t="n">
         <v>215</v>
       </c>
-      <c r="I35" t="n">
+      <c r="I35" s="18" t="n">
         <v>112</v>
       </c>
-      <c r="J35" t="n">
+      <c r="J35" s="18" t="n">
         <v>1769</v>
       </c>
-      <c r="K35" t="n">
+      <c r="K35" s="18" t="n">
         <v>6.33</v>
       </c>
-      <c r="L35" t="n">
+      <c r="L35" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="M35" t="n">
+      <c r="M35" s="18" t="n">
         <v>140</v>
       </c>
-      <c r="N35" t="n">
+      <c r="N35" s="18" t="n">
         <v>186</v>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="O35" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-26.csv</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="19">
-      <c r="A36" s="22" t="n"/>
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>76</v>
+      </c>
+      <c r="C36" t="n">
+        <v>74</v>
+      </c>
+      <c r="D36" t="n">
+        <v>64443</v>
+      </c>
+      <c r="E36" t="n">
+        <v>463476</v>
+      </c>
+      <c r="F36" t="n">
+        <v>13.78</v>
+      </c>
+      <c r="G36" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H36" t="n">
+        <v>218</v>
+      </c>
+      <c r="I36" t="n">
+        <v>111</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1825</v>
+      </c>
+      <c r="K36" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="L36" t="n">
+        <v>18</v>
+      </c>
+      <c r="M36" t="n">
+        <v>143</v>
+      </c>
+      <c r="N36" t="n">
+        <v>190</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-27.csv</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="19">
       <c r="A37" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-28
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2327,53 +2327,101 @@
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D36" t="n">
+      <c r="D36" s="18" t="n">
         <v>64443</v>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="18" t="n">
         <v>463476</v>
       </c>
-      <c r="F36" t="n">
+      <c r="F36" s="18" t="n">
         <v>13.78</v>
       </c>
-      <c r="G36" t="n">
+      <c r="G36" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H36" t="n">
+      <c r="H36" s="18" t="n">
         <v>218</v>
       </c>
-      <c r="I36" t="n">
+      <c r="I36" s="18" t="n">
         <v>111</v>
       </c>
-      <c r="J36" t="n">
+      <c r="J36" s="18" t="n">
         <v>1825</v>
       </c>
-      <c r="K36" t="n">
+      <c r="K36" s="18" t="n">
         <v>6.08</v>
       </c>
-      <c r="L36" t="n">
+      <c r="L36" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="M36" t="n">
+      <c r="M36" s="18" t="n">
         <v>143</v>
       </c>
-      <c r="N36" t="n">
+      <c r="N36" s="18" t="n">
         <v>190</v>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="O36" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-27.csv</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="19">
-      <c r="A37" s="22" t="n"/>
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>76</v>
+      </c>
+      <c r="C37" t="n">
+        <v>74</v>
+      </c>
+      <c r="D37" t="n">
+        <v>64267</v>
+      </c>
+      <c r="E37" t="n">
+        <v>461695</v>
+      </c>
+      <c r="F37" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="G37" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H37" t="n">
+        <v>221</v>
+      </c>
+      <c r="I37" t="n">
+        <v>116</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1860</v>
+      </c>
+      <c r="K37" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="L37" t="n">
+        <v>17</v>
+      </c>
+      <c r="M37" t="n">
+        <v>145</v>
+      </c>
+      <c r="N37" t="n">
+        <v>194</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-28.csv</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="19">
       <c r="A38" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-29
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2378,53 +2378,101 @@
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D37" t="n">
+      <c r="D37" s="18" t="n">
         <v>64267</v>
       </c>
-      <c r="E37" t="n">
+      <c r="E37" s="18" t="n">
         <v>461695</v>
       </c>
-      <c r="F37" t="n">
+      <c r="F37" s="18" t="n">
         <v>13.8</v>
       </c>
-      <c r="G37" t="n">
+      <c r="G37" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H37" t="n">
+      <c r="H37" s="18" t="n">
         <v>221</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I37" s="18" t="n">
         <v>116</v>
       </c>
-      <c r="J37" t="n">
+      <c r="J37" s="18" t="n">
         <v>1860</v>
       </c>
-      <c r="K37" t="n">
+      <c r="K37" s="18" t="n">
         <v>6.24</v>
       </c>
-      <c r="L37" t="n">
+      <c r="L37" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="M37" t="n">
+      <c r="M37" s="18" t="n">
         <v>145</v>
       </c>
-      <c r="N37" t="n">
+      <c r="N37" s="18" t="n">
         <v>194</v>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="O37" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-28.csv</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="19">
-      <c r="A38" s="22" t="n"/>
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>76</v>
+      </c>
+      <c r="C38" t="n">
+        <v>74</v>
+      </c>
+      <c r="D38" t="n">
+        <v>64218</v>
+      </c>
+      <c r="E38" t="n">
+        <v>461486</v>
+      </c>
+      <c r="F38" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="G38" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="H38" t="n">
+        <v>225</v>
+      </c>
+      <c r="I38" t="n">
+        <v>116</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1886</v>
+      </c>
+      <c r="K38" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="L38" t="n">
+        <v>18</v>
+      </c>
+      <c r="M38" t="n">
+        <v>148</v>
+      </c>
+      <c r="N38" t="n">
+        <v>197</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-29.csv</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="19">
       <c r="A39" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-06-30
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2429,53 +2429,101 @@
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D38" s="18" t="n">
         <v>64218</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E38" s="18" t="n">
         <v>461486</v>
       </c>
-      <c r="F38" t="n">
+      <c r="F38" s="18" t="n">
         <v>13.8</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G38" s="18" t="n">
         <v>47.4</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H38" s="18" t="n">
         <v>225</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I38" s="18" t="n">
         <v>116</v>
       </c>
-      <c r="J38" t="n">
+      <c r="J38" s="18" t="n">
         <v>1886</v>
       </c>
-      <c r="K38" t="n">
+      <c r="K38" s="18" t="n">
         <v>6.15</v>
       </c>
-      <c r="L38" t="n">
+      <c r="L38" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="M38" t="n">
+      <c r="M38" s="18" t="n">
         <v>148</v>
       </c>
-      <c r="N38" t="n">
+      <c r="N38" s="18" t="n">
         <v>197</v>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="O38" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-29.csv</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="19">
-      <c r="A39" s="22" t="n"/>
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>76</v>
+      </c>
+      <c r="C39" t="n">
+        <v>74</v>
+      </c>
+      <c r="D39" t="n">
+        <v>60351</v>
+      </c>
+      <c r="E39" t="n">
+        <v>447942</v>
+      </c>
+      <c r="F39" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="G39" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H39" t="n">
+        <v>227</v>
+      </c>
+      <c r="I39" t="n">
+        <v>124</v>
+      </c>
+      <c r="J39" t="n">
+        <v>1925</v>
+      </c>
+      <c r="K39" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="L39" t="n">
+        <v>19</v>
+      </c>
+      <c r="M39" t="n">
+        <v>151</v>
+      </c>
+      <c r="N39" t="n">
+        <v>199</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-06-30.csv</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="19">
       <c r="A40" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-01
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2480,53 +2480,101 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="18" t="n">
         <v>60351</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="18" t="n">
         <v>447942</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="18" t="n">
         <v>13.35</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G39" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="18" t="n">
         <v>227</v>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" s="18" t="n">
         <v>124</v>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" s="18" t="n">
         <v>1925</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K39" s="18" t="n">
         <v>6.44</v>
       </c>
-      <c r="L39" t="n">
+      <c r="L39" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="M39" t="n">
+      <c r="M39" s="18" t="n">
         <v>151</v>
       </c>
-      <c r="N39" t="n">
+      <c r="N39" s="18" t="n">
         <v>199</v>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="O39" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-06-30.csv</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="19">
-      <c r="A40" s="22" t="n"/>
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>76</v>
+      </c>
+      <c r="C40" t="n">
+        <v>74</v>
+      </c>
+      <c r="D40" t="n">
+        <v>52257</v>
+      </c>
+      <c r="E40" t="n">
+        <v>412388</v>
+      </c>
+      <c r="F40" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="G40" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>230</v>
+      </c>
+      <c r="I40" t="n">
+        <v>123</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1997</v>
+      </c>
+      <c r="K40" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="L40" t="n">
+        <v>19</v>
+      </c>
+      <c r="M40" t="n">
+        <v>157</v>
+      </c>
+      <c r="N40" t="n">
+        <v>204</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-01.csv</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="19">
       <c r="A41" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-02
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2531,53 +2531,101 @@
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D40" s="18" t="n">
         <v>52257</v>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="18" t="n">
         <v>412388</v>
       </c>
-      <c r="F40" t="n">
+      <c r="F40" s="18" t="n">
         <v>12.54</v>
       </c>
-      <c r="G40" t="n">
+      <c r="G40" s="18" t="n">
         <v>47.2</v>
       </c>
-      <c r="H40" t="n">
+      <c r="H40" s="18" t="n">
         <v>230</v>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" s="18" t="n">
         <v>123</v>
       </c>
-      <c r="J40" t="n">
+      <c r="J40" s="18" t="n">
         <v>1997</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K40" s="18" t="n">
         <v>6.16</v>
       </c>
-      <c r="L40" t="n">
+      <c r="L40" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="M40" t="n">
+      <c r="M40" s="18" t="n">
         <v>157</v>
       </c>
-      <c r="N40" t="n">
+      <c r="N40" s="18" t="n">
         <v>204</v>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="O40" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-01.csv</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="19">
-      <c r="A41" s="22" t="n"/>
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>76</v>
+      </c>
+      <c r="C41" t="n">
+        <v>74</v>
+      </c>
+      <c r="D41" t="n">
+        <v>44115</v>
+      </c>
+      <c r="E41" t="n">
+        <v>388373</v>
+      </c>
+      <c r="F41" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="G41" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="H41" t="n">
+        <v>237</v>
+      </c>
+      <c r="I41" t="n">
+        <v>122</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2106</v>
+      </c>
+      <c r="K41" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="L41" t="n">
+        <v>20</v>
+      </c>
+      <c r="M41" t="n">
+        <v>159</v>
+      </c>
+      <c r="N41" t="n">
+        <v>215</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-02.csv</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="19">
       <c r="A42" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-03
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2582,53 +2582,101 @@
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D41" t="n">
+      <c r="D41" s="18" t="n">
         <v>44115</v>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="18" t="n">
         <v>388373</v>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" s="18" t="n">
         <v>11.21</v>
       </c>
-      <c r="G41" t="n">
+      <c r="G41" s="18" t="n">
         <v>47.4</v>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="18" t="n">
         <v>237</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I41" s="18" t="n">
         <v>122</v>
       </c>
-      <c r="J41" t="n">
+      <c r="J41" s="18" t="n">
         <v>2106</v>
       </c>
-      <c r="K41" t="n">
+      <c r="K41" s="18" t="n">
         <v>5.79</v>
       </c>
-      <c r="L41" t="n">
+      <c r="L41" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M41" t="n">
+      <c r="M41" s="18" t="n">
         <v>159</v>
       </c>
-      <c r="N41" t="n">
+      <c r="N41" s="18" t="n">
         <v>215</v>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="O41" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-02.csv</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="19">
-      <c r="A42" s="22" t="n"/>
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>76</v>
+      </c>
+      <c r="C42" t="n">
+        <v>74</v>
+      </c>
+      <c r="D42" t="n">
+        <v>39239</v>
+      </c>
+      <c r="E42" t="n">
+        <v>374795</v>
+      </c>
+      <c r="F42" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="G42" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H42" t="n">
+        <v>241</v>
+      </c>
+      <c r="I42" t="n">
+        <v>122</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2196</v>
+      </c>
+      <c r="K42" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="L42" t="n">
+        <v>22</v>
+      </c>
+      <c r="M42" t="n">
+        <v>162</v>
+      </c>
+      <c r="N42" t="n">
+        <v>215</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-03.csv</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="19">
       <c r="A43" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-04
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2633,53 +2633,101 @@
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D42" t="n">
+      <c r="D42" s="18" t="n">
         <v>39239</v>
       </c>
-      <c r="E42" t="n">
+      <c r="E42" s="18" t="n">
         <v>374795</v>
       </c>
-      <c r="F42" t="n">
+      <c r="F42" s="18" t="n">
         <v>10.32</v>
       </c>
-      <c r="G42" t="n">
+      <c r="G42" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H42" t="n">
+      <c r="H42" s="18" t="n">
         <v>241</v>
       </c>
-      <c r="I42" t="n">
+      <c r="I42" s="18" t="n">
         <v>122</v>
       </c>
-      <c r="J42" t="n">
+      <c r="J42" s="18" t="n">
         <v>2196</v>
       </c>
-      <c r="K42" t="n">
+      <c r="K42" s="18" t="n">
         <v>5.56</v>
       </c>
-      <c r="L42" t="n">
+      <c r="L42" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M42" t="n">
+      <c r="M42" s="18" t="n">
         <v>162</v>
       </c>
-      <c r="N42" t="n">
+      <c r="N42" s="18" t="n">
         <v>215</v>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="O42" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-03.csv</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="19">
-      <c r="A43" s="22" t="n"/>
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>76</v>
+      </c>
+      <c r="C43" t="n">
+        <v>74</v>
+      </c>
+      <c r="D43" t="n">
+        <v>36940</v>
+      </c>
+      <c r="E43" t="n">
+        <v>366435</v>
+      </c>
+      <c r="F43" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="G43" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H43" t="n">
+        <v>241</v>
+      </c>
+      <c r="I43" t="n">
+        <v>121</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2284</v>
+      </c>
+      <c r="K43" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="L43" t="n">
+        <v>22</v>
+      </c>
+      <c r="M43" t="n">
+        <v>158</v>
+      </c>
+      <c r="N43" t="n">
+        <v>214</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-04.csv</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="19">
       <c r="A44" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-05
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2684,53 +2684,101 @@
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D43" t="n">
+      <c r="D43" s="18" t="n">
         <v>36940</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="18" t="n">
         <v>366435</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" s="18" t="n">
         <v>9.93</v>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" s="18" t="n">
         <v>47.6</v>
       </c>
-      <c r="H43" t="n">
+      <c r="H43" s="18" t="n">
         <v>241</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" s="18" t="n">
         <v>121</v>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" s="18" t="n">
         <v>2284</v>
       </c>
-      <c r="K43" t="n">
+      <c r="K43" s="18" t="n">
         <v>5.3</v>
       </c>
-      <c r="L43" t="n">
+      <c r="L43" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M43" t="n">
+      <c r="M43" s="18" t="n">
         <v>158</v>
       </c>
-      <c r="N43" t="n">
+      <c r="N43" s="18" t="n">
         <v>214</v>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="O43" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-04.csv</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="19">
-      <c r="A44" s="22" t="n"/>
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>76</v>
+      </c>
+      <c r="C44" t="n">
+        <v>74</v>
+      </c>
+      <c r="D44" t="n">
+        <v>35531</v>
+      </c>
+      <c r="E44" t="n">
+        <v>362117</v>
+      </c>
+      <c r="F44" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="G44" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="H44" t="n">
+        <v>245</v>
+      </c>
+      <c r="I44" t="n">
+        <v>120</v>
+      </c>
+      <c r="J44" t="n">
+        <v>2338</v>
+      </c>
+      <c r="K44" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="L44" t="n">
+        <v>21</v>
+      </c>
+      <c r="M44" t="n">
+        <v>163</v>
+      </c>
+      <c r="N44" t="n">
+        <v>218</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-05.csv</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="19">
       <c r="A45" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-06
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2735,53 +2735,101 @@
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D44" t="n">
+      <c r="D44" s="18" t="n">
         <v>35531</v>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="18" t="n">
         <v>362117</v>
       </c>
-      <c r="F44" t="n">
+      <c r="F44" s="18" t="n">
         <v>9.66</v>
       </c>
-      <c r="G44" t="n">
+      <c r="G44" s="18" t="n">
         <v>47.7</v>
       </c>
-      <c r="H44" t="n">
+      <c r="H44" s="18" t="n">
         <v>245</v>
       </c>
-      <c r="I44" t="n">
+      <c r="I44" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="J44" t="n">
+      <c r="J44" s="18" t="n">
         <v>2338</v>
       </c>
-      <c r="K44" t="n">
+      <c r="K44" s="18" t="n">
         <v>5.13</v>
       </c>
-      <c r="L44" t="n">
+      <c r="L44" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="M44" t="n">
+      <c r="M44" s="18" t="n">
         <v>163</v>
       </c>
-      <c r="N44" t="n">
+      <c r="N44" s="18" t="n">
         <v>218</v>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="O44" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-05.csv</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="19">
-      <c r="A45" s="22" t="n"/>
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>76</v>
+      </c>
+      <c r="C45" t="n">
+        <v>74</v>
+      </c>
+      <c r="D45" t="n">
+        <v>34771</v>
+      </c>
+      <c r="E45" t="n">
+        <v>358658</v>
+      </c>
+      <c r="F45" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="G45" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H45" t="n">
+        <v>248</v>
+      </c>
+      <c r="I45" t="n">
+        <v>125</v>
+      </c>
+      <c r="J45" t="n">
+        <v>2405</v>
+      </c>
+      <c r="K45" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="L45" t="n">
+        <v>22</v>
+      </c>
+      <c r="M45" t="n">
+        <v>164</v>
+      </c>
+      <c r="N45" t="n">
+        <v>220</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-06.csv</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="19">
       <c r="A46" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-07
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2786,53 +2786,101 @@
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D45" s="18" t="n">
         <v>34771</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="18" t="n">
         <v>358658</v>
       </c>
-      <c r="F45" t="n">
+      <c r="F45" s="18" t="n">
         <v>9.539999999999999</v>
       </c>
-      <c r="G45" t="n">
+      <c r="G45" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H45" t="n">
+      <c r="H45" s="18" t="n">
         <v>248</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I45" s="18" t="n">
         <v>125</v>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" s="18" t="n">
         <v>2405</v>
       </c>
-      <c r="K45" t="n">
+      <c r="K45" s="18" t="n">
         <v>5.2</v>
       </c>
-      <c r="L45" t="n">
+      <c r="L45" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M45" t="n">
+      <c r="M45" s="18" t="n">
         <v>164</v>
       </c>
-      <c r="N45" t="n">
+      <c r="N45" s="18" t="n">
         <v>220</v>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="O45" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-06.csv</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="19">
-      <c r="A46" s="22" t="n"/>
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>76</v>
+      </c>
+      <c r="C46" t="n">
+        <v>74</v>
+      </c>
+      <c r="D46" t="n">
+        <v>30824</v>
+      </c>
+      <c r="E46" t="n">
+        <v>320844</v>
+      </c>
+      <c r="F46" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="G46" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H46" t="n">
+        <v>252</v>
+      </c>
+      <c r="I46" t="n">
+        <v>124</v>
+      </c>
+      <c r="J46" t="n">
+        <v>2469</v>
+      </c>
+      <c r="K46" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="L46" t="n">
+        <v>22</v>
+      </c>
+      <c r="M46" t="n">
+        <v>165</v>
+      </c>
+      <c r="N46" t="n">
+        <v>223</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-07.csv</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="19">
       <c r="A47" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-08
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2837,53 +2837,101 @@
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D46" t="n">
+      <c r="D46" s="18" t="n">
         <v>30824</v>
       </c>
-      <c r="E46" t="n">
+      <c r="E46" s="18" t="n">
         <v>320844</v>
       </c>
-      <c r="F46" t="n">
+      <c r="F46" s="18" t="n">
         <v>9.43</v>
       </c>
-      <c r="G46" t="n">
+      <c r="G46" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H46" t="n">
+      <c r="H46" s="18" t="n">
         <v>252</v>
       </c>
-      <c r="I46" t="n">
+      <c r="I46" s="18" t="n">
         <v>124</v>
       </c>
-      <c r="J46" t="n">
+      <c r="J46" s="18" t="n">
         <v>2469</v>
       </c>
-      <c r="K46" t="n">
+      <c r="K46" s="18" t="n">
         <v>5.02</v>
       </c>
-      <c r="L46" t="n">
+      <c r="L46" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M46" t="n">
+      <c r="M46" s="18" t="n">
         <v>165</v>
       </c>
-      <c r="N46" t="n">
+      <c r="N46" s="18" t="n">
         <v>223</v>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="O46" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-07.csv</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="19">
-      <c r="A47" s="22" t="n"/>
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>76</v>
+      </c>
+      <c r="C47" t="n">
+        <v>74</v>
+      </c>
+      <c r="D47" t="n">
+        <v>27328</v>
+      </c>
+      <c r="E47" t="n">
+        <v>286690</v>
+      </c>
+      <c r="F47" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="G47" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H47" t="n">
+        <v>262</v>
+      </c>
+      <c r="I47" t="n">
+        <v>129</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2594</v>
+      </c>
+      <c r="K47" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="L47" t="n">
+        <v>23</v>
+      </c>
+      <c r="M47" t="n">
+        <v>171</v>
+      </c>
+      <c r="N47" t="n">
+        <v>231</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-08.csv</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="19">
       <c r="A48" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-09
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2888,53 +2888,101 @@
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C47" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D47" t="n">
+      <c r="D47" s="18" t="n">
         <v>27328</v>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="18" t="n">
         <v>286690</v>
       </c>
-      <c r="F47" t="n">
+      <c r="F47" s="18" t="n">
         <v>9.34</v>
       </c>
-      <c r="G47" t="n">
+      <c r="G47" s="18" t="n">
         <v>47.6</v>
       </c>
-      <c r="H47" t="n">
+      <c r="H47" s="18" t="n">
         <v>262</v>
       </c>
-      <c r="I47" t="n">
+      <c r="I47" s="18" t="n">
         <v>129</v>
       </c>
-      <c r="J47" t="n">
+      <c r="J47" s="18" t="n">
         <v>2594</v>
       </c>
-      <c r="K47" t="n">
+      <c r="K47" s="18" t="n">
         <v>4.97</v>
       </c>
-      <c r="L47" t="n">
+      <c r="L47" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="M47" t="n">
+      <c r="M47" s="18" t="n">
         <v>171</v>
       </c>
-      <c r="N47" t="n">
+      <c r="N47" s="18" t="n">
         <v>231</v>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O47" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-08.csv</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="19">
-      <c r="A48" s="22" t="n"/>
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>76</v>
+      </c>
+      <c r="C48" t="n">
+        <v>74</v>
+      </c>
+      <c r="D48" t="n">
+        <v>22528</v>
+      </c>
+      <c r="E48" t="n">
+        <v>242926</v>
+      </c>
+      <c r="F48" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="G48" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H48" t="n">
+        <v>269</v>
+      </c>
+      <c r="I48" t="n">
+        <v>129</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2695</v>
+      </c>
+      <c r="K48" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="L48" t="n">
+        <v>22</v>
+      </c>
+      <c r="M48" t="n">
+        <v>171</v>
+      </c>
+      <c r="N48" t="n">
+        <v>236</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-09.csv</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="19">
       <c r="A49" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-10
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2939,53 +2939,101 @@
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C48" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D48" t="n">
+      <c r="D48" s="18" t="n">
         <v>22528</v>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="18" t="n">
         <v>242926</v>
       </c>
-      <c r="F48" t="n">
+      <c r="F48" s="18" t="n">
         <v>9.039999999999999</v>
       </c>
-      <c r="G48" t="n">
+      <c r="G48" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H48" t="n">
+      <c r="H48" s="18" t="n">
         <v>269</v>
       </c>
-      <c r="I48" t="n">
+      <c r="I48" s="18" t="n">
         <v>129</v>
       </c>
-      <c r="J48" t="n">
+      <c r="J48" s="18" t="n">
         <v>2695</v>
       </c>
-      <c r="K48" t="n">
+      <c r="K48" s="18" t="n">
         <v>4.79</v>
       </c>
-      <c r="L48" t="n">
+      <c r="L48" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M48" t="n">
+      <c r="M48" s="18" t="n">
         <v>171</v>
       </c>
-      <c r="N48" t="n">
+      <c r="N48" s="18" t="n">
         <v>236</v>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="O48" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-09.csv</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="19">
-      <c r="A49" s="22" t="n"/>
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>76</v>
+      </c>
+      <c r="C49" t="n">
+        <v>74</v>
+      </c>
+      <c r="D49" t="n">
+        <v>19228</v>
+      </c>
+      <c r="E49" t="n">
+        <v>214121</v>
+      </c>
+      <c r="F49" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G49" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="H49" t="n">
+        <v>270</v>
+      </c>
+      <c r="I49" t="n">
+        <v>132</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2786</v>
+      </c>
+      <c r="K49" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="L49" t="n">
+        <v>23</v>
+      </c>
+      <c r="M49" t="n">
+        <v>170</v>
+      </c>
+      <c r="N49" t="n">
+        <v>235</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-10.csv</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="19">
       <c r="A50" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-11
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -2990,53 +2990,101 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C49" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D49" t="n">
+      <c r="D49" s="18" t="n">
         <v>19228</v>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="18" t="n">
         <v>214121</v>
       </c>
-      <c r="F49" t="n">
+      <c r="F49" s="18" t="n">
         <v>8.720000000000001</v>
       </c>
-      <c r="G49" t="n">
+      <c r="G49" s="18" t="n">
         <v>47.1</v>
       </c>
-      <c r="H49" t="n">
+      <c r="H49" s="18" t="n">
         <v>270</v>
       </c>
-      <c r="I49" t="n">
+      <c r="I49" s="18" t="n">
         <v>132</v>
       </c>
-      <c r="J49" t="n">
+      <c r="J49" s="18" t="n">
         <v>2786</v>
       </c>
-      <c r="K49" t="n">
+      <c r="K49" s="18" t="n">
         <v>4.74</v>
       </c>
-      <c r="L49" t="n">
+      <c r="L49" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="M49" t="n">
+      <c r="M49" s="18" t="n">
         <v>170</v>
       </c>
-      <c r="N49" t="n">
+      <c r="N49" s="18" t="n">
         <v>235</v>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="O49" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-10.csv</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="19">
-      <c r="A50" s="22" t="n"/>
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>76</v>
+      </c>
+      <c r="C50" t="n">
+        <v>74</v>
+      </c>
+      <c r="D50" t="n">
+        <v>17351</v>
+      </c>
+      <c r="E50" t="n">
+        <v>199846</v>
+      </c>
+      <c r="F50" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G50" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H50" t="n">
+        <v>268</v>
+      </c>
+      <c r="I50" t="n">
+        <v>131</v>
+      </c>
+      <c r="J50" t="n">
+        <v>2855</v>
+      </c>
+      <c r="K50" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="L50" t="n">
+        <v>21</v>
+      </c>
+      <c r="M50" t="n">
+        <v>163</v>
+      </c>
+      <c r="N50" t="n">
+        <v>232</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-11.csv</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="19">
       <c r="A51" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-12
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3041,53 +3041,101 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C50" t="n">
+      <c r="C50" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D50" t="n">
+      <c r="D50" s="18" t="n">
         <v>17351</v>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="18" t="n">
         <v>199846</v>
       </c>
-      <c r="F50" t="n">
+      <c r="F50" s="18" t="n">
         <v>8.4</v>
       </c>
-      <c r="G50" t="n">
+      <c r="G50" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H50" t="n">
+      <c r="H50" s="18" t="n">
         <v>268</v>
       </c>
-      <c r="I50" t="n">
+      <c r="I50" s="18" t="n">
         <v>131</v>
       </c>
-      <c r="J50" t="n">
+      <c r="J50" s="18" t="n">
         <v>2855</v>
       </c>
-      <c r="K50" t="n">
+      <c r="K50" s="18" t="n">
         <v>4.59</v>
       </c>
-      <c r="L50" t="n">
+      <c r="L50" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="M50" t="n">
+      <c r="M50" s="18" t="n">
         <v>163</v>
       </c>
-      <c r="N50" t="n">
+      <c r="N50" s="18" t="n">
         <v>232</v>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="O50" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-11.csv</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="19">
-      <c r="A51" s="22" t="n"/>
+      <c r="A51" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>76</v>
+      </c>
+      <c r="C51" t="n">
+        <v>74</v>
+      </c>
+      <c r="D51" t="n">
+        <v>16463</v>
+      </c>
+      <c r="E51" t="n">
+        <v>190641</v>
+      </c>
+      <c r="F51" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="G51" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H51" t="n">
+        <v>270</v>
+      </c>
+      <c r="I51" t="n">
+        <v>132</v>
+      </c>
+      <c r="J51" t="n">
+        <v>2963</v>
+      </c>
+      <c r="K51" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="L51" t="n">
+        <v>22</v>
+      </c>
+      <c r="M51" t="n">
+        <v>164</v>
+      </c>
+      <c r="N51" t="n">
+        <v>231</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-12.csv</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="19">
       <c r="A52" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-13
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3092,53 +3092,101 @@
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C51" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D51" t="n">
+      <c r="D51" s="18" t="n">
         <v>16463</v>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="18" t="n">
         <v>190641</v>
       </c>
-      <c r="F51" t="n">
+      <c r="F51" s="18" t="n">
         <v>8.34</v>
       </c>
-      <c r="G51" t="n">
+      <c r="G51" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H51" t="n">
+      <c r="H51" s="18" t="n">
         <v>270</v>
       </c>
-      <c r="I51" t="n">
+      <c r="I51" s="18" t="n">
         <v>132</v>
       </c>
-      <c r="J51" t="n">
+      <c r="J51" s="18" t="n">
         <v>2963</v>
       </c>
-      <c r="K51" t="n">
+      <c r="K51" s="18" t="n">
         <v>4.45</v>
       </c>
-      <c r="L51" t="n">
+      <c r="L51" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M51" t="n">
+      <c r="M51" s="18" t="n">
         <v>164</v>
       </c>
-      <c r="N51" t="n">
+      <c r="N51" s="18" t="n">
         <v>231</v>
       </c>
-      <c r="O51" t="inlineStr">
+      <c r="O51" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-12.csv</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="19">
-      <c r="A52" s="22" t="n"/>
+      <c r="A52" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>76</v>
+      </c>
+      <c r="C52" t="n">
+        <v>74</v>
+      </c>
+      <c r="D52" t="n">
+        <v>15938</v>
+      </c>
+      <c r="E52" t="n">
+        <v>185192</v>
+      </c>
+      <c r="F52" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G52" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H52" t="n">
+        <v>277</v>
+      </c>
+      <c r="I52" t="n">
+        <v>135</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3080</v>
+      </c>
+      <c r="K52" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="L52" t="n">
+        <v>21</v>
+      </c>
+      <c r="M52" t="n">
+        <v>170</v>
+      </c>
+      <c r="N52" t="n">
+        <v>238</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-13.csv</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="19">
       <c r="A53" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-14
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3143,53 +3143,101 @@
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B52" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C52" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D52" t="n">
+      <c r="D52" s="18" t="n">
         <v>15938</v>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="18" t="n">
         <v>185192</v>
       </c>
-      <c r="F52" t="n">
+      <c r="F52" s="18" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G52" t="n">
+      <c r="G52" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H52" t="n">
+      <c r="H52" s="18" t="n">
         <v>277</v>
       </c>
-      <c r="I52" t="n">
+      <c r="I52" s="18" t="n">
         <v>135</v>
       </c>
-      <c r="J52" t="n">
+      <c r="J52" s="18" t="n">
         <v>3080</v>
       </c>
-      <c r="K52" t="n">
+      <c r="K52" s="18" t="n">
         <v>4.38</v>
       </c>
-      <c r="L52" t="n">
+      <c r="L52" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="M52" t="n">
+      <c r="M52" s="18" t="n">
         <v>170</v>
       </c>
-      <c r="N52" t="n">
+      <c r="N52" s="18" t="n">
         <v>238</v>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="O52" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-13.csv</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="19">
-      <c r="A53" s="22" t="n"/>
+      <c r="A53" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>76</v>
+      </c>
+      <c r="C53" t="n">
+        <v>74</v>
+      </c>
+      <c r="D53" t="n">
+        <v>15659</v>
+      </c>
+      <c r="E53" t="n">
+        <v>182288</v>
+      </c>
+      <c r="F53" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="G53" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H53" t="n">
+        <v>277</v>
+      </c>
+      <c r="I53" t="n">
+        <v>130</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3155</v>
+      </c>
+      <c r="K53" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="L53" t="n">
+        <v>20</v>
+      </c>
+      <c r="M53" t="n">
+        <v>170</v>
+      </c>
+      <c r="N53" t="n">
+        <v>237</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-14.csv</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="19">
       <c r="A54" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-15
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3194,53 +3194,101 @@
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B53" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C53" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D53" t="n">
+      <c r="D53" s="18" t="n">
         <v>15659</v>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="18" t="n">
         <v>182288</v>
       </c>
-      <c r="F53" t="n">
+      <c r="F53" s="18" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="G53" t="n">
+      <c r="G53" s="18" t="n">
         <v>47.3</v>
       </c>
-      <c r="H53" t="n">
+      <c r="H53" s="18" t="n">
         <v>277</v>
       </c>
-      <c r="I53" t="n">
+      <c r="I53" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="J53" t="n">
+      <c r="J53" s="18" t="n">
         <v>3155</v>
       </c>
-      <c r="K53" t="n">
+      <c r="K53" s="18" t="n">
         <v>4.12</v>
       </c>
-      <c r="L53" t="n">
+      <c r="L53" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M53" t="n">
+      <c r="M53" s="18" t="n">
         <v>170</v>
       </c>
-      <c r="N53" t="n">
+      <c r="N53" s="18" t="n">
         <v>237</v>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="O53" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-14.csv</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="19">
-      <c r="A54" s="22" t="n"/>
+      <c r="A54" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>76</v>
+      </c>
+      <c r="C54" t="n">
+        <v>74</v>
+      </c>
+      <c r="D54" t="n">
+        <v>15426</v>
+      </c>
+      <c r="E54" t="n">
+        <v>179201</v>
+      </c>
+      <c r="F54" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G54" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>282</v>
+      </c>
+      <c r="I54" t="n">
+        <v>130</v>
+      </c>
+      <c r="J54" t="n">
+        <v>3247</v>
+      </c>
+      <c r="K54" t="n">
+        <v>4</v>
+      </c>
+      <c r="L54" t="n">
+        <v>20</v>
+      </c>
+      <c r="M54" t="n">
+        <v>171</v>
+      </c>
+      <c r="N54" t="n">
+        <v>242</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-15.csv</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="19">
       <c r="A55" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-16
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3245,53 +3245,101 @@
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B54" t="n">
+      <c r="B54" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D54" t="n">
+      <c r="D54" s="18" t="n">
         <v>15426</v>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="18" t="n">
         <v>179201</v>
       </c>
-      <c r="F54" t="n">
+      <c r="F54" s="18" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G54" t="n">
+      <c r="G54" s="18" t="n">
         <v>47.1</v>
       </c>
-      <c r="H54" t="n">
+      <c r="H54" s="18" t="n">
         <v>282</v>
       </c>
-      <c r="I54" t="n">
+      <c r="I54" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="J54" t="n">
+      <c r="J54" s="18" t="n">
         <v>3247</v>
       </c>
-      <c r="K54" t="n">
+      <c r="K54" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="L54" t="n">
+      <c r="L54" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M54" t="n">
+      <c r="M54" s="18" t="n">
         <v>171</v>
       </c>
-      <c r="N54" t="n">
+      <c r="N54" s="18" t="n">
         <v>242</v>
       </c>
-      <c r="O54" t="inlineStr">
+      <c r="O54" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-15.csv</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="19">
-      <c r="A55" s="22" t="n"/>
+      <c r="A55" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>76</v>
+      </c>
+      <c r="C55" t="n">
+        <v>74</v>
+      </c>
+      <c r="D55" t="n">
+        <v>15240</v>
+      </c>
+      <c r="E55" t="n">
+        <v>176797</v>
+      </c>
+      <c r="F55" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G55" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="H55" t="n">
+        <v>278</v>
+      </c>
+      <c r="I55" t="n">
+        <v>124</v>
+      </c>
+      <c r="J55" t="n">
+        <v>3280</v>
+      </c>
+      <c r="K55" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="L55" t="n">
+        <v>20</v>
+      </c>
+      <c r="M55" t="n">
+        <v>170</v>
+      </c>
+      <c r="N55" t="n">
+        <v>240</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-16.csv</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="19">
       <c r="A56" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-17
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3296,53 +3296,101 @@
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B55" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D55" t="n">
+      <c r="D55" s="18" t="n">
         <v>15240</v>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="18" t="n">
         <v>176797</v>
       </c>
-      <c r="F55" t="n">
+      <c r="F55" s="18" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G55" t="n">
+      <c r="G55" s="18" t="n">
         <v>47.2</v>
       </c>
-      <c r="H55" t="n">
+      <c r="H55" s="18" t="n">
         <v>278</v>
       </c>
-      <c r="I55" t="n">
+      <c r="I55" s="18" t="n">
         <v>124</v>
       </c>
-      <c r="J55" t="n">
+      <c r="J55" s="18" t="n">
         <v>3280</v>
       </c>
-      <c r="K55" t="n">
+      <c r="K55" s="18" t="n">
         <v>3.78</v>
       </c>
-      <c r="L55" t="n">
+      <c r="L55" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M55" t="n">
+      <c r="M55" s="18" t="n">
         <v>170</v>
       </c>
-      <c r="N55" t="n">
+      <c r="N55" s="18" t="n">
         <v>240</v>
       </c>
-      <c r="O55" t="inlineStr">
+      <c r="O55" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-16.csv</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="19">
-      <c r="A56" s="22" t="n"/>
+      <c r="A56" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>76</v>
+      </c>
+      <c r="C56" t="n">
+        <v>74</v>
+      </c>
+      <c r="D56" t="n">
+        <v>15009</v>
+      </c>
+      <c r="E56" t="n">
+        <v>173993</v>
+      </c>
+      <c r="F56" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G56" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="H56" t="n">
+        <v>275</v>
+      </c>
+      <c r="I56" t="n">
+        <v>121</v>
+      </c>
+      <c r="J56" t="n">
+        <v>3361</v>
+      </c>
+      <c r="K56" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L56" t="n">
+        <v>19</v>
+      </c>
+      <c r="M56" t="n">
+        <v>167</v>
+      </c>
+      <c r="N56" t="n">
+        <v>235</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-17.csv</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="19">
       <c r="A57" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-18
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3347,53 +3347,101 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B56" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D56" t="n">
+      <c r="D56" s="18" t="n">
         <v>15009</v>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="18" t="n">
         <v>173993</v>
       </c>
-      <c r="F56" t="n">
+      <c r="F56" s="18" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G56" t="n">
+      <c r="G56" s="18" t="n">
         <v>46.7</v>
       </c>
-      <c r="H56" t="n">
+      <c r="H56" s="18" t="n">
         <v>275</v>
       </c>
-      <c r="I56" t="n">
+      <c r="I56" s="18" t="n">
         <v>121</v>
       </c>
-      <c r="J56" t="n">
+      <c r="J56" s="18" t="n">
         <v>3361</v>
       </c>
-      <c r="K56" t="n">
+      <c r="K56" s="18" t="n">
         <v>3.6</v>
       </c>
-      <c r="L56" t="n">
+      <c r="L56" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="M56" t="n">
+      <c r="M56" s="18" t="n">
         <v>167</v>
       </c>
-      <c r="N56" t="n">
+      <c r="N56" s="18" t="n">
         <v>235</v>
       </c>
-      <c r="O56" t="inlineStr">
+      <c r="O56" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-17.csv</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="19">
-      <c r="A57" s="22" t="n"/>
+      <c r="A57" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>76</v>
+      </c>
+      <c r="C57" t="n">
+        <v>74</v>
+      </c>
+      <c r="D57" t="n">
+        <v>14818</v>
+      </c>
+      <c r="E57" t="n">
+        <v>171564</v>
+      </c>
+      <c r="F57" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="G57" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="H57" t="n">
+        <v>274</v>
+      </c>
+      <c r="I57" t="n">
+        <v>124</v>
+      </c>
+      <c r="J57" t="n">
+        <v>3433</v>
+      </c>
+      <c r="K57" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="L57" t="n">
+        <v>18</v>
+      </c>
+      <c r="M57" t="n">
+        <v>165</v>
+      </c>
+      <c r="N57" t="n">
+        <v>233</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-18.csv</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="19">
       <c r="A58" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-19
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3398,53 +3398,101 @@
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="B57" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C57" t="n">
+      <c r="C57" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D57" t="n">
+      <c r="D57" s="18" t="n">
         <v>14818</v>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="18" t="n">
         <v>171564</v>
       </c>
-      <c r="F57" t="n">
+      <c r="F57" s="18" t="n">
         <v>8.31</v>
       </c>
-      <c r="G57" t="n">
+      <c r="G57" s="18" t="n">
         <v>46.7</v>
       </c>
-      <c r="H57" t="n">
+      <c r="H57" s="18" t="n">
         <v>274</v>
       </c>
-      <c r="I57" t="n">
+      <c r="I57" s="18" t="n">
         <v>124</v>
       </c>
-      <c r="J57" t="n">
+      <c r="J57" s="18" t="n">
         <v>3433</v>
       </c>
-      <c r="K57" t="n">
+      <c r="K57" s="18" t="n">
         <v>3.61</v>
       </c>
-      <c r="L57" t="n">
+      <c r="L57" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="M57" t="n">
+      <c r="M57" s="18" t="n">
         <v>165</v>
       </c>
-      <c r="N57" t="n">
+      <c r="N57" s="18" t="n">
         <v>233</v>
       </c>
-      <c r="O57" t="inlineStr">
+      <c r="O57" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-18.csv</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="19">
-      <c r="A58" s="22" t="n"/>
+      <c r="A58" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>78</v>
+      </c>
+      <c r="C58" t="n">
+        <v>74</v>
+      </c>
+      <c r="D58" t="n">
+        <v>14704</v>
+      </c>
+      <c r="E58" t="n">
+        <v>170190</v>
+      </c>
+      <c r="F58" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="G58" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="H58" t="n">
+        <v>276</v>
+      </c>
+      <c r="I58" t="n">
+        <v>127</v>
+      </c>
+      <c r="J58" t="n">
+        <v>3545</v>
+      </c>
+      <c r="K58" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="L58" t="n">
+        <v>18</v>
+      </c>
+      <c r="M58" t="n">
+        <v>166</v>
+      </c>
+      <c r="N58" t="n">
+        <v>237</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-19.csv</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="19">
       <c r="A59" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-20
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3449,53 +3449,101 @@
           <t>2026-07-19</t>
         </is>
       </c>
-      <c r="B58" t="n">
+      <c r="B58" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="C58" t="n">
+      <c r="C58" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D58" t="n">
+      <c r="D58" s="18" t="n">
         <v>14704</v>
       </c>
-      <c r="E58" t="n">
+      <c r="E58" s="18" t="n">
         <v>170190</v>
       </c>
-      <c r="F58" t="n">
+      <c r="F58" s="18" t="n">
         <v>8.31</v>
       </c>
-      <c r="G58" t="n">
+      <c r="G58" s="18" t="n">
         <v>46.9</v>
       </c>
-      <c r="H58" t="n">
+      <c r="H58" s="18" t="n">
         <v>276</v>
       </c>
-      <c r="I58" t="n">
+      <c r="I58" s="18" t="n">
         <v>127</v>
       </c>
-      <c r="J58" t="n">
+      <c r="J58" s="18" t="n">
         <v>3545</v>
       </c>
-      <c r="K58" t="n">
+      <c r="K58" s="18" t="n">
         <v>3.58</v>
       </c>
-      <c r="L58" t="n">
+      <c r="L58" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="M58" t="n">
+      <c r="M58" s="18" t="n">
         <v>166</v>
       </c>
-      <c r="N58" t="n">
+      <c r="N58" s="18" t="n">
         <v>237</v>
       </c>
-      <c r="O58" t="inlineStr">
+      <c r="O58" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-19.csv</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="19">
-      <c r="A59" s="22" t="n"/>
+      <c r="A59" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>78</v>
+      </c>
+      <c r="C59" t="n">
+        <v>74</v>
+      </c>
+      <c r="D59" t="n">
+        <v>14567</v>
+      </c>
+      <c r="E59" t="n">
+        <v>168924</v>
+      </c>
+      <c r="F59" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="G59" t="n">
+        <v>47</v>
+      </c>
+      <c r="H59" t="n">
+        <v>287</v>
+      </c>
+      <c r="I59" t="n">
+        <v>129</v>
+      </c>
+      <c r="J59" t="n">
+        <v>3627</v>
+      </c>
+      <c r="K59" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="L59" t="n">
+        <v>20</v>
+      </c>
+      <c r="M59" t="n">
+        <v>177</v>
+      </c>
+      <c r="N59" t="n">
+        <v>246</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-20.csv</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="19">
       <c r="A60" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-21
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3500,53 +3500,101 @@
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="B59" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="D59" t="n">
+      <c r="D59" s="18" t="n">
         <v>14567</v>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="18" t="n">
         <v>168924</v>
       </c>
-      <c r="F59" t="n">
+      <c r="F59" s="18" t="n">
         <v>8.289999999999999</v>
       </c>
-      <c r="G59" t="n">
+      <c r="G59" s="18" t="n">
         <v>47</v>
       </c>
-      <c r="H59" t="n">
+      <c r="H59" s="18" t="n">
         <v>287</v>
       </c>
-      <c r="I59" t="n">
+      <c r="I59" s="18" t="n">
         <v>129</v>
       </c>
-      <c r="J59" t="n">
+      <c r="J59" s="18" t="n">
         <v>3627</v>
       </c>
-      <c r="K59" t="n">
+      <c r="K59" s="18" t="n">
         <v>3.56</v>
       </c>
-      <c r="L59" t="n">
+      <c r="L59" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M59" t="n">
+      <c r="M59" s="18" t="n">
         <v>177</v>
       </c>
-      <c r="N59" t="n">
+      <c r="N59" s="18" t="n">
         <v>246</v>
       </c>
-      <c r="O59" t="inlineStr">
+      <c r="O59" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-20.csv</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="19">
-      <c r="A60" s="22" t="n"/>
+      <c r="A60" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>79</v>
+      </c>
+      <c r="C60" t="n">
+        <v>76</v>
+      </c>
+      <c r="D60" t="n">
+        <v>14612</v>
+      </c>
+      <c r="E60" t="n">
+        <v>168798</v>
+      </c>
+      <c r="F60" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="G60" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="H60" t="n">
+        <v>292</v>
+      </c>
+      <c r="I60" t="n">
+        <v>130</v>
+      </c>
+      <c r="J60" t="n">
+        <v>3739</v>
+      </c>
+      <c r="K60" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="L60" t="n">
+        <v>20</v>
+      </c>
+      <c r="M60" t="n">
+        <v>177</v>
+      </c>
+      <c r="N60" t="n">
+        <v>250</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-21.csv</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="19">
       <c r="A61" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-22
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3551,53 +3551,101 @@
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="B60" t="n">
+      <c r="B60" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="D60" t="n">
+      <c r="D60" s="18" t="n">
         <v>14612</v>
       </c>
-      <c r="E60" t="n">
+      <c r="E60" s="18" t="n">
         <v>168798</v>
       </c>
-      <c r="F60" t="n">
+      <c r="F60" s="18" t="n">
         <v>8.32</v>
       </c>
-      <c r="G60" t="n">
+      <c r="G60" s="18" t="n">
         <v>47.4</v>
       </c>
-      <c r="H60" t="n">
+      <c r="H60" s="18" t="n">
         <v>292</v>
       </c>
-      <c r="I60" t="n">
+      <c r="I60" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="J60" t="n">
+      <c r="J60" s="18" t="n">
         <v>3739</v>
       </c>
-      <c r="K60" t="n">
+      <c r="K60" s="18" t="n">
         <v>3.48</v>
       </c>
-      <c r="L60" t="n">
+      <c r="L60" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M60" t="n">
+      <c r="M60" s="18" t="n">
         <v>177</v>
       </c>
-      <c r="N60" t="n">
+      <c r="N60" s="18" t="n">
         <v>250</v>
       </c>
-      <c r="O60" t="inlineStr">
+      <c r="O60" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-21.csv</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="19">
-      <c r="A61" s="22" t="n"/>
+      <c r="A61" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>79</v>
+      </c>
+      <c r="C61" t="n">
+        <v>76</v>
+      </c>
+      <c r="D61" t="n">
+        <v>16702</v>
+      </c>
+      <c r="E61" t="n">
+        <v>180235</v>
+      </c>
+      <c r="F61" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="G61" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="H61" t="n">
+        <v>295</v>
+      </c>
+      <c r="I61" t="n">
+        <v>136</v>
+      </c>
+      <c r="J61" t="n">
+        <v>3851</v>
+      </c>
+      <c r="K61" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="L61" t="n">
+        <v>20</v>
+      </c>
+      <c r="M61" t="n">
+        <v>178</v>
+      </c>
+      <c r="N61" t="n">
+        <v>253</v>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-22.csv</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="19">
       <c r="A62" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-23
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3602,53 +3602,101 @@
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="B61" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C61" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="D61" t="n">
+      <c r="D61" s="18" t="n">
         <v>16702</v>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="18" t="n">
         <v>180235</v>
       </c>
-      <c r="F61" t="n">
+      <c r="F61" s="18" t="n">
         <v>8.960000000000001</v>
       </c>
-      <c r="G61" t="n">
+      <c r="G61" s="18" t="n">
         <v>47.4</v>
       </c>
-      <c r="H61" t="n">
+      <c r="H61" s="18" t="n">
         <v>295</v>
       </c>
-      <c r="I61" t="n">
+      <c r="I61" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="J61" t="n">
+      <c r="J61" s="18" t="n">
         <v>3851</v>
       </c>
-      <c r="K61" t="n">
+      <c r="K61" s="18" t="n">
         <v>3.53</v>
       </c>
-      <c r="L61" t="n">
+      <c r="L61" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M61" t="n">
+      <c r="M61" s="18" t="n">
         <v>178</v>
       </c>
-      <c r="N61" t="n">
+      <c r="N61" s="18" t="n">
         <v>253</v>
       </c>
-      <c r="O61" t="inlineStr">
+      <c r="O61" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-22.csv</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="19">
-      <c r="A62" s="22" t="n"/>
+      <c r="A62" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>79</v>
+      </c>
+      <c r="C62" t="n">
+        <v>77</v>
+      </c>
+      <c r="D62" t="n">
+        <v>16916</v>
+      </c>
+      <c r="E62" t="n">
+        <v>179464</v>
+      </c>
+      <c r="F62" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="G62" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="H62" t="n">
+        <v>294</v>
+      </c>
+      <c r="I62" t="n">
+        <v>130</v>
+      </c>
+      <c r="J62" t="n">
+        <v>3884</v>
+      </c>
+      <c r="K62" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="L62" t="n">
+        <v>17</v>
+      </c>
+      <c r="M62" t="n">
+        <v>182</v>
+      </c>
+      <c r="N62" t="n">
+        <v>253</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-23.csv</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="19">
       <c r="A63" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-24
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3653,53 +3653,101 @@
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="B62" t="n">
+      <c r="B62" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" s="18" t="n">
         <v>77</v>
       </c>
-      <c r="D62" t="n">
+      <c r="D62" s="18" t="n">
         <v>16916</v>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="18" t="n">
         <v>179464</v>
       </c>
-      <c r="F62" t="n">
+      <c r="F62" s="18" t="n">
         <v>9.109999999999999</v>
       </c>
-      <c r="G62" t="n">
+      <c r="G62" s="18" t="n">
         <v>47.7</v>
       </c>
-      <c r="H62" t="n">
+      <c r="H62" s="18" t="n">
         <v>294</v>
       </c>
-      <c r="I62" t="n">
+      <c r="I62" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="J62" t="n">
+      <c r="J62" s="18" t="n">
         <v>3884</v>
       </c>
-      <c r="K62" t="n">
+      <c r="K62" s="18" t="n">
         <v>3.35</v>
       </c>
-      <c r="L62" t="n">
+      <c r="L62" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="M62" t="n">
+      <c r="M62" s="18" t="n">
         <v>182</v>
       </c>
-      <c r="N62" t="n">
+      <c r="N62" s="18" t="n">
         <v>253</v>
       </c>
-      <c r="O62" t="inlineStr">
+      <c r="O62" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-23.csv</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="19">
-      <c r="A63" s="22" t="n"/>
+      <c r="A63" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>80</v>
+      </c>
+      <c r="C63" t="n">
+        <v>77</v>
+      </c>
+      <c r="D63" t="n">
+        <v>16956</v>
+      </c>
+      <c r="E63" t="n">
+        <v>177933</v>
+      </c>
+      <c r="F63" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="G63" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H63" t="n">
+        <v>298</v>
+      </c>
+      <c r="I63" t="n">
+        <v>130</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3931</v>
+      </c>
+      <c r="K63" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="L63" t="n">
+        <v>16</v>
+      </c>
+      <c r="M63" t="n">
+        <v>183</v>
+      </c>
+      <c r="N63" t="n">
+        <v>257</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-24.csv</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="19">
       <c r="A64" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-25
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3704,53 +3704,101 @@
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="B63" t="n">
+      <c r="B63" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" s="18" t="n">
         <v>77</v>
       </c>
-      <c r="D63" t="n">
+      <c r="D63" s="18" t="n">
         <v>16956</v>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="18" t="n">
         <v>177933</v>
       </c>
-      <c r="F63" t="n">
+      <c r="F63" s="18" t="n">
         <v>9.210000000000001</v>
       </c>
-      <c r="G63" t="n">
+      <c r="G63" s="18" t="n">
         <v>47.6</v>
       </c>
-      <c r="H63" t="n">
+      <c r="H63" s="18" t="n">
         <v>298</v>
       </c>
-      <c r="I63" t="n">
+      <c r="I63" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="J63" t="n">
+      <c r="J63" s="18" t="n">
         <v>3931</v>
       </c>
-      <c r="K63" t="n">
+      <c r="K63" s="18" t="n">
         <v>3.31</v>
       </c>
-      <c r="L63" t="n">
+      <c r="L63" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="M63" t="n">
+      <c r="M63" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="N63" t="n">
+      <c r="N63" s="18" t="n">
         <v>257</v>
       </c>
-      <c r="O63" t="inlineStr">
+      <c r="O63" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-24.csv</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="19">
-      <c r="A64" s="22" t="n"/>
+      <c r="A64" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>80</v>
+      </c>
+      <c r="C64" t="n">
+        <v>77</v>
+      </c>
+      <c r="D64" t="n">
+        <v>17017</v>
+      </c>
+      <c r="E64" t="n">
+        <v>179038</v>
+      </c>
+      <c r="F64" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="G64" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H64" t="n">
+        <v>299</v>
+      </c>
+      <c r="I64" t="n">
+        <v>132</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3986</v>
+      </c>
+      <c r="K64" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="L64" t="n">
+        <v>17</v>
+      </c>
+      <c r="M64" t="n">
+        <v>180</v>
+      </c>
+      <c r="N64" t="n">
+        <v>258</v>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-25.csv</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="19">
       <c r="A65" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-26
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3755,53 +3755,101 @@
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="B64" t="n">
+      <c r="B64" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C64" t="n">
+      <c r="C64" s="18" t="n">
         <v>77</v>
       </c>
-      <c r="D64" t="n">
+      <c r="D64" s="18" t="n">
         <v>17017</v>
       </c>
-      <c r="E64" t="n">
+      <c r="E64" s="18" t="n">
         <v>179038</v>
       </c>
-      <c r="F64" t="n">
+      <c r="F64" s="18" t="n">
         <v>9.19</v>
       </c>
-      <c r="G64" t="n">
+      <c r="G64" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H64" t="n">
+      <c r="H64" s="18" t="n">
         <v>299</v>
       </c>
-      <c r="I64" t="n">
+      <c r="I64" s="18" t="n">
         <v>132</v>
       </c>
-      <c r="J64" t="n">
+      <c r="J64" s="18" t="n">
         <v>3986</v>
       </c>
-      <c r="K64" t="n">
+      <c r="K64" s="18" t="n">
         <v>3.31</v>
       </c>
-      <c r="L64" t="n">
+      <c r="L64" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="M64" t="n">
+      <c r="M64" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="N64" t="n">
+      <c r="N64" s="18" t="n">
         <v>258</v>
       </c>
-      <c r="O64" t="inlineStr">
+      <c r="O64" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-25.csv</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="19">
-      <c r="A65" s="22" t="n"/>
+      <c r="A65" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>80</v>
+      </c>
+      <c r="C65" t="n">
+        <v>78</v>
+      </c>
+      <c r="D65" t="n">
+        <v>19328</v>
+      </c>
+      <c r="E65" t="n">
+        <v>190913</v>
+      </c>
+      <c r="F65" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="G65" t="n">
+        <v>48</v>
+      </c>
+      <c r="H65" t="n">
+        <v>304</v>
+      </c>
+      <c r="I65" t="n">
+        <v>127</v>
+      </c>
+      <c r="J65" t="n">
+        <v>4088</v>
+      </c>
+      <c r="K65" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="L65" t="n">
+        <v>18</v>
+      </c>
+      <c r="M65" t="n">
+        <v>183</v>
+      </c>
+      <c r="N65" t="n">
+        <v>260</v>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-26.csv</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="19">
       <c r="A66" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-27
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3806,53 +3806,101 @@
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="B65" t="n">
+      <c r="B65" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C65" t="n">
+      <c r="C65" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D65" t="n">
+      <c r="D65" s="18" t="n">
         <v>19328</v>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="18" t="n">
         <v>190913</v>
       </c>
-      <c r="F65" t="n">
+      <c r="F65" s="18" t="n">
         <v>9.83</v>
       </c>
-      <c r="G65" t="n">
+      <c r="G65" s="18" t="n">
         <v>48</v>
       </c>
-      <c r="H65" t="n">
+      <c r="H65" s="18" t="n">
         <v>304</v>
       </c>
-      <c r="I65" t="n">
+      <c r="I65" s="18" t="n">
         <v>127</v>
       </c>
-      <c r="J65" t="n">
+      <c r="J65" s="18" t="n">
         <v>4088</v>
       </c>
-      <c r="K65" t="n">
+      <c r="K65" s="18" t="n">
         <v>3.11</v>
       </c>
-      <c r="L65" t="n">
+      <c r="L65" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="M65" t="n">
+      <c r="M65" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="N65" t="n">
+      <c r="N65" s="18" t="n">
         <v>260</v>
       </c>
-      <c r="O65" t="inlineStr">
+      <c r="O65" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-26.csv</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="19">
-      <c r="A66" s="22" t="n"/>
+      <c r="A66" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>80</v>
+      </c>
+      <c r="C66" t="n">
+        <v>78</v>
+      </c>
+      <c r="D66" t="n">
+        <v>22093</v>
+      </c>
+      <c r="E66" t="n">
+        <v>207126</v>
+      </c>
+      <c r="F66" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G66" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="H66" t="n">
+        <v>307</v>
+      </c>
+      <c r="I66" t="n">
+        <v>127</v>
+      </c>
+      <c r="J66" t="n">
+        <v>4161</v>
+      </c>
+      <c r="K66" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="L66" t="n">
+        <v>17</v>
+      </c>
+      <c r="M66" t="n">
+        <v>185</v>
+      </c>
+      <c r="N66" t="n">
+        <v>261</v>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-27.csv</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="19">
       <c r="A67" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-28
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3857,53 +3857,101 @@
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="B66" t="n">
+      <c r="B66" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C66" t="n">
+      <c r="C66" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D66" t="n">
+      <c r="D66" s="18" t="n">
         <v>22093</v>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="18" t="n">
         <v>207126</v>
       </c>
-      <c r="F66" t="n">
+      <c r="F66" s="18" t="n">
         <v>10.4</v>
       </c>
-      <c r="G66" t="n">
+      <c r="G66" s="18" t="n">
         <v>47.8</v>
       </c>
-      <c r="H66" t="n">
+      <c r="H66" s="18" t="n">
         <v>307</v>
       </c>
-      <c r="I66" t="n">
+      <c r="I66" s="18" t="n">
         <v>127</v>
       </c>
-      <c r="J66" t="n">
+      <c r="J66" s="18" t="n">
         <v>4161</v>
       </c>
-      <c r="K66" t="n">
+      <c r="K66" s="18" t="n">
         <v>3.05</v>
       </c>
-      <c r="L66" t="n">
+      <c r="L66" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="M66" t="n">
+      <c r="M66" s="18" t="n">
         <v>185</v>
       </c>
-      <c r="N66" t="n">
+      <c r="N66" s="18" t="n">
         <v>261</v>
       </c>
-      <c r="O66" t="inlineStr">
+      <c r="O66" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-27.csv</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="19">
-      <c r="A67" s="22" t="n"/>
+      <c r="A67" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>80</v>
+      </c>
+      <c r="C67" t="n">
+        <v>78</v>
+      </c>
+      <c r="D67" t="n">
+        <v>24714</v>
+      </c>
+      <c r="E67" t="n">
+        <v>223165</v>
+      </c>
+      <c r="F67" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="G67" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H67" t="n">
+        <v>315</v>
+      </c>
+      <c r="I67" t="n">
+        <v>121</v>
+      </c>
+      <c r="J67" t="n">
+        <v>4232</v>
+      </c>
+      <c r="K67" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="L67" t="n">
+        <v>17</v>
+      </c>
+      <c r="M67" t="n">
+        <v>187</v>
+      </c>
+      <c r="N67" t="n">
+        <v>265</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-28.csv</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="19">
       <c r="A68" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-29
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3908,53 +3908,101 @@
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B67" t="n">
+      <c r="B67" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C67" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D67" t="n">
+      <c r="D67" s="18" t="n">
         <v>24714</v>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="18" t="n">
         <v>223165</v>
       </c>
-      <c r="F67" t="n">
+      <c r="F67" s="18" t="n">
         <v>10.82</v>
       </c>
-      <c r="G67" t="n">
+      <c r="G67" s="18" t="n">
         <v>47.6</v>
       </c>
-      <c r="H67" t="n">
+      <c r="H67" s="18" t="n">
         <v>315</v>
       </c>
-      <c r="I67" t="n">
+      <c r="I67" s="18" t="n">
         <v>121</v>
       </c>
-      <c r="J67" t="n">
+      <c r="J67" s="18" t="n">
         <v>4232</v>
       </c>
-      <c r="K67" t="n">
+      <c r="K67" s="18" t="n">
         <v>2.86</v>
       </c>
-      <c r="L67" t="n">
+      <c r="L67" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="M67" t="n">
+      <c r="M67" s="18" t="n">
         <v>187</v>
       </c>
-      <c r="N67" t="n">
+      <c r="N67" s="18" t="n">
         <v>265</v>
       </c>
-      <c r="O67" t="inlineStr">
+      <c r="O67" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-28.csv</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="19">
-      <c r="A68" s="22" t="n"/>
+      <c r="A68" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>80</v>
+      </c>
+      <c r="C68" t="n">
+        <v>78</v>
+      </c>
+      <c r="D68" t="n">
+        <v>26407</v>
+      </c>
+      <c r="E68" t="n">
+        <v>234228</v>
+      </c>
+      <c r="F68" t="n">
+        <v>11.03</v>
+      </c>
+      <c r="G68" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H68" t="n">
+        <v>318</v>
+      </c>
+      <c r="I68" t="n">
+        <v>117</v>
+      </c>
+      <c r="J68" t="n">
+        <v>4315</v>
+      </c>
+      <c r="K68" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="L68" t="n">
+        <v>19</v>
+      </c>
+      <c r="M68" t="n">
+        <v>184</v>
+      </c>
+      <c r="N68" t="n">
+        <v>264</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-29.csv</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="19">
       <c r="A69" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-30
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -3959,53 +3959,101 @@
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B68" t="n">
+      <c r="B68" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C68" t="n">
+      <c r="C68" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D68" t="n">
+      <c r="D68" s="18" t="n">
         <v>26407</v>
       </c>
-      <c r="E68" t="n">
+      <c r="E68" s="18" t="n">
         <v>234228</v>
       </c>
-      <c r="F68" t="n">
+      <c r="F68" s="18" t="n">
         <v>11.03</v>
       </c>
-      <c r="G68" t="n">
+      <c r="G68" s="18" t="n">
         <v>47.5</v>
       </c>
-      <c r="H68" t="n">
+      <c r="H68" s="18" t="n">
         <v>318</v>
       </c>
-      <c r="I68" t="n">
+      <c r="I68" s="18" t="n">
         <v>117</v>
       </c>
-      <c r="J68" t="n">
+      <c r="J68" s="18" t="n">
         <v>4315</v>
       </c>
-      <c r="K68" t="n">
+      <c r="K68" s="18" t="n">
         <v>2.71</v>
       </c>
-      <c r="L68" t="n">
+      <c r="L68" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="M68" t="n">
+      <c r="M68" s="18" t="n">
         <v>184</v>
       </c>
-      <c r="N68" t="n">
+      <c r="N68" s="18" t="n">
         <v>264</v>
       </c>
-      <c r="O68" t="inlineStr">
+      <c r="O68" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-29.csv</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="19">
-      <c r="A69" s="22" t="n"/>
+      <c r="A69" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>80</v>
+      </c>
+      <c r="C69" t="n">
+        <v>78</v>
+      </c>
+      <c r="D69" t="n">
+        <v>27627</v>
+      </c>
+      <c r="E69" t="n">
+        <v>242296</v>
+      </c>
+      <c r="F69" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="G69" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="H69" t="n">
+        <v>322</v>
+      </c>
+      <c r="I69" t="n">
+        <v>115</v>
+      </c>
+      <c r="J69" t="n">
+        <v>4321</v>
+      </c>
+      <c r="K69" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L69" t="n">
+        <v>18</v>
+      </c>
+      <c r="M69" t="n">
+        <v>183</v>
+      </c>
+      <c r="N69" t="n">
+        <v>266</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-30.csv</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="19">
       <c r="A70" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-07-31
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4010,53 +4010,101 @@
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B69" t="n">
+      <c r="B69" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D69" t="n">
+      <c r="D69" s="18" t="n">
         <v>27627</v>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="18" t="n">
         <v>242296</v>
       </c>
-      <c r="F69" t="n">
+      <c r="F69" s="18" t="n">
         <v>11.17</v>
       </c>
-      <c r="G69" t="n">
+      <c r="G69" s="18" t="n">
         <v>48.7</v>
       </c>
-      <c r="H69" t="n">
+      <c r="H69" s="18" t="n">
         <v>322</v>
       </c>
-      <c r="I69" t="n">
+      <c r="I69" s="18" t="n">
         <v>115</v>
       </c>
-      <c r="J69" t="n">
+      <c r="J69" s="18" t="n">
         <v>4321</v>
       </c>
-      <c r="K69" t="n">
+      <c r="K69" s="18" t="n">
         <v>2.66</v>
       </c>
-      <c r="L69" t="n">
+      <c r="L69" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="M69" t="n">
+      <c r="M69" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="N69" t="n">
+      <c r="N69" s="18" t="n">
         <v>266</v>
       </c>
-      <c r="O69" t="inlineStr">
+      <c r="O69" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-30.csv</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="19">
-      <c r="A70" s="22" t="n"/>
+      <c r="A70" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>80</v>
+      </c>
+      <c r="C70" t="n">
+        <v>78</v>
+      </c>
+      <c r="D70" t="n">
+        <v>28552</v>
+      </c>
+      <c r="E70" t="n">
+        <v>247641</v>
+      </c>
+      <c r="F70" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G70" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="H70" t="n">
+        <v>324</v>
+      </c>
+      <c r="I70" t="n">
+        <v>113</v>
+      </c>
+      <c r="J70" t="n">
+        <v>4351</v>
+      </c>
+      <c r="K70" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L70" t="n">
+        <v>21</v>
+      </c>
+      <c r="M70" t="n">
+        <v>183</v>
+      </c>
+      <c r="N70" t="n">
+        <v>267</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-07-31.csv</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="19">
       <c r="A71" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-01
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4061,53 +4061,101 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B70" t="n">
+      <c r="B70" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D70" t="n">
+      <c r="D70" s="18" t="n">
         <v>28552</v>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="18" t="n">
         <v>247641</v>
       </c>
-      <c r="F70" t="n">
+      <c r="F70" s="18" t="n">
         <v>11.3</v>
       </c>
-      <c r="G70" t="n">
+      <c r="G70" s="18" t="n">
         <v>48.6</v>
       </c>
-      <c r="H70" t="n">
+      <c r="H70" s="18" t="n">
         <v>324</v>
       </c>
-      <c r="I70" t="n">
+      <c r="I70" s="18" t="n">
         <v>113</v>
       </c>
-      <c r="J70" t="n">
+      <c r="J70" s="18" t="n">
         <v>4351</v>
       </c>
-      <c r="K70" t="n">
+      <c r="K70" s="18" t="n">
         <v>2.6</v>
       </c>
-      <c r="L70" t="n">
+      <c r="L70" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="M70" t="n">
+      <c r="M70" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="N70" t="n">
+      <c r="N70" s="18" t="n">
         <v>267</v>
       </c>
-      <c r="O70" t="inlineStr">
+      <c r="O70" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-07-31.csv</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="19">
-      <c r="A71" s="22" t="n"/>
+      <c r="A71" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>80</v>
+      </c>
+      <c r="C71" t="n">
+        <v>78</v>
+      </c>
+      <c r="D71" t="n">
+        <v>29023</v>
+      </c>
+      <c r="E71" t="n">
+        <v>250510</v>
+      </c>
+      <c r="F71" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="G71" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="H71" t="n">
+        <v>335</v>
+      </c>
+      <c r="I71" t="n">
+        <v>114</v>
+      </c>
+      <c r="J71" t="n">
+        <v>4437</v>
+      </c>
+      <c r="K71" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="L71" t="n">
+        <v>20</v>
+      </c>
+      <c r="M71" t="n">
+        <v>188</v>
+      </c>
+      <c r="N71" t="n">
+        <v>273</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-01.csv</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="19">
       <c r="A72" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-02
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4112,53 +4112,101 @@
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="B71" t="n">
+      <c r="B71" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D71" t="n">
+      <c r="D71" s="18" t="n">
         <v>29023</v>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="18" t="n">
         <v>250510</v>
       </c>
-      <c r="F71" t="n">
+      <c r="F71" s="18" t="n">
         <v>11.36</v>
       </c>
-      <c r="G71" t="n">
+      <c r="G71" s="18" t="n">
         <v>48.5</v>
       </c>
-      <c r="H71" t="n">
+      <c r="H71" s="18" t="n">
         <v>335</v>
       </c>
-      <c r="I71" t="n">
+      <c r="I71" s="18" t="n">
         <v>114</v>
       </c>
-      <c r="J71" t="n">
+      <c r="J71" s="18" t="n">
         <v>4437</v>
       </c>
-      <c r="K71" t="n">
+      <c r="K71" s="18" t="n">
         <v>2.57</v>
       </c>
-      <c r="L71" t="n">
+      <c r="L71" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="M71" t="n">
+      <c r="M71" s="18" t="n">
         <v>188</v>
       </c>
-      <c r="N71" t="n">
+      <c r="N71" s="18" t="n">
         <v>273</v>
       </c>
-      <c r="O71" t="inlineStr">
+      <c r="O71" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-01.csv</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="19">
-      <c r="A72" s="22" t="n"/>
+      <c r="A72" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>80</v>
+      </c>
+      <c r="C72" t="n">
+        <v>78</v>
+      </c>
+      <c r="D72" t="n">
+        <v>29623</v>
+      </c>
+      <c r="E72" t="n">
+        <v>253211</v>
+      </c>
+      <c r="F72" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="G72" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="H72" t="n">
+        <v>344</v>
+      </c>
+      <c r="I72" t="n">
+        <v>114</v>
+      </c>
+      <c r="J72" t="n">
+        <v>4504</v>
+      </c>
+      <c r="K72" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="L72" t="n">
+        <v>21</v>
+      </c>
+      <c r="M72" t="n">
+        <v>189</v>
+      </c>
+      <c r="N72" t="n">
+        <v>279</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-02.csv</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="19">
       <c r="A73" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-03
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4163,53 +4163,101 @@
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="B72" t="n">
+      <c r="B72" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D72" t="n">
+      <c r="D72" s="18" t="n">
         <v>29623</v>
       </c>
-      <c r="E72" t="n">
+      <c r="E72" s="18" t="n">
         <v>253211</v>
       </c>
-      <c r="F72" t="n">
+      <c r="F72" s="18" t="n">
         <v>11.48</v>
       </c>
-      <c r="G72" t="n">
+      <c r="G72" s="18" t="n">
         <v>48.4</v>
       </c>
-      <c r="H72" t="n">
+      <c r="H72" s="18" t="n">
         <v>344</v>
       </c>
-      <c r="I72" t="n">
+      <c r="I72" s="18" t="n">
         <v>114</v>
       </c>
-      <c r="J72" t="n">
+      <c r="J72" s="18" t="n">
         <v>4504</v>
       </c>
-      <c r="K72" t="n">
+      <c r="K72" s="18" t="n">
         <v>2.53</v>
       </c>
-      <c r="L72" t="n">
+      <c r="L72" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="M72" t="n">
+      <c r="M72" s="18" t="n">
         <v>189</v>
       </c>
-      <c r="N72" t="n">
+      <c r="N72" s="18" t="n">
         <v>279</v>
       </c>
-      <c r="O72" t="inlineStr">
+      <c r="O72" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-02.csv</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="19">
-      <c r="A73" s="22" t="n"/>
+      <c r="A73" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>80</v>
+      </c>
+      <c r="C73" t="n">
+        <v>78</v>
+      </c>
+      <c r="D73" t="n">
+        <v>29972</v>
+      </c>
+      <c r="E73" t="n">
+        <v>255345</v>
+      </c>
+      <c r="F73" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="G73" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="H73" t="n">
+        <v>347</v>
+      </c>
+      <c r="I73" t="n">
+        <v>113</v>
+      </c>
+      <c r="J73" t="n">
+        <v>4602</v>
+      </c>
+      <c r="K73" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="L73" t="n">
+        <v>22</v>
+      </c>
+      <c r="M73" t="n">
+        <v>188</v>
+      </c>
+      <c r="N73" t="n">
+        <v>280</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-03.csv</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="19">
       <c r="A74" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-04
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4214,53 +4214,101 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B73" t="n">
+      <c r="B73" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D73" t="n">
+      <c r="D73" s="18" t="n">
         <v>29972</v>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="18" t="n">
         <v>255345</v>
       </c>
-      <c r="F73" t="n">
+      <c r="F73" s="18" t="n">
         <v>11.52</v>
       </c>
-      <c r="G73" t="n">
+      <c r="G73" s="18" t="n">
         <v>48.4</v>
       </c>
-      <c r="H73" t="n">
+      <c r="H73" s="18" t="n">
         <v>347</v>
       </c>
-      <c r="I73" t="n">
+      <c r="I73" s="18" t="n">
         <v>113</v>
       </c>
-      <c r="J73" t="n">
+      <c r="J73" s="18" t="n">
         <v>4602</v>
       </c>
-      <c r="K73" t="n">
+      <c r="K73" s="18" t="n">
         <v>2.46</v>
       </c>
-      <c r="L73" t="n">
+      <c r="L73" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="M73" t="n">
+      <c r="M73" s="18" t="n">
         <v>188</v>
       </c>
-      <c r="N73" t="n">
+      <c r="N73" s="18" t="n">
         <v>280</v>
       </c>
-      <c r="O73" t="inlineStr">
+      <c r="O73" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-03.csv</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="19">
-      <c r="A74" s="22" t="n"/>
+      <c r="A74" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>80</v>
+      </c>
+      <c r="C74" t="n">
+        <v>78</v>
+      </c>
+      <c r="D74" t="n">
+        <v>30264</v>
+      </c>
+      <c r="E74" t="n">
+        <v>257506</v>
+      </c>
+      <c r="F74" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="G74" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="H74" t="n">
+        <v>352</v>
+      </c>
+      <c r="I74" t="n">
+        <v>113</v>
+      </c>
+      <c r="J74" t="n">
+        <v>4686</v>
+      </c>
+      <c r="K74" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="L74" t="n">
+        <v>23</v>
+      </c>
+      <c r="M74" t="n">
+        <v>189</v>
+      </c>
+      <c r="N74" t="n">
+        <v>283</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-04.csv</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="19">
       <c r="A75" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-05
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4265,53 +4265,101 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="B74" t="n">
+      <c r="B74" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C74" t="n">
+      <c r="C74" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D74" t="n">
+      <c r="D74" s="18" t="n">
         <v>30264</v>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="18" t="n">
         <v>257506</v>
       </c>
-      <c r="F74" t="n">
+      <c r="F74" s="18" t="n">
         <v>11.54</v>
       </c>
-      <c r="G74" t="n">
+      <c r="G74" s="18" t="n">
         <v>48.4</v>
       </c>
-      <c r="H74" t="n">
+      <c r="H74" s="18" t="n">
         <v>352</v>
       </c>
-      <c r="I74" t="n">
+      <c r="I74" s="18" t="n">
         <v>113</v>
       </c>
-      <c r="J74" t="n">
+      <c r="J74" s="18" t="n">
         <v>4686</v>
       </c>
-      <c r="K74" t="n">
+      <c r="K74" s="18" t="n">
         <v>2.41</v>
       </c>
-      <c r="L74" t="n">
+      <c r="L74" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="M74" t="n">
+      <c r="M74" s="18" t="n">
         <v>189</v>
       </c>
-      <c r="N74" t="n">
+      <c r="N74" s="18" t="n">
         <v>283</v>
       </c>
-      <c r="O74" t="inlineStr">
+      <c r="O74" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-04.csv</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="19">
-      <c r="A75" s="22" t="n"/>
+      <c r="A75" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>80</v>
+      </c>
+      <c r="C75" t="n">
+        <v>78</v>
+      </c>
+      <c r="D75" t="n">
+        <v>30357</v>
+      </c>
+      <c r="E75" t="n">
+        <v>258127</v>
+      </c>
+      <c r="F75" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="G75" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="H75" t="n">
+        <v>364</v>
+      </c>
+      <c r="I75" t="n">
+        <v>108</v>
+      </c>
+      <c r="J75" t="n">
+        <v>4660</v>
+      </c>
+      <c r="K75" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="L75" t="n">
+        <v>25</v>
+      </c>
+      <c r="M75" t="n">
+        <v>196</v>
+      </c>
+      <c r="N75" t="n">
+        <v>293</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-05.csv</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="19">
       <c r="A76" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-06
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4316,53 +4316,101 @@
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B75" t="n">
+      <c r="B75" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="18" t="n">
         <v>30357</v>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="18" t="n">
         <v>258127</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="18" t="n">
         <v>11.54</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G75" s="18" t="n">
         <v>48.4</v>
       </c>
-      <c r="H75" t="n">
+      <c r="H75" s="18" t="n">
         <v>364</v>
       </c>
-      <c r="I75" t="n">
+      <c r="I75" s="18" t="n">
         <v>108</v>
       </c>
-      <c r="J75" t="n">
+      <c r="J75" s="18" t="n">
         <v>4660</v>
       </c>
-      <c r="K75" t="n">
+      <c r="K75" s="18" t="n">
         <v>2.32</v>
       </c>
-      <c r="L75" t="n">
+      <c r="L75" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="M75" t="n">
+      <c r="M75" s="18" t="n">
         <v>196</v>
       </c>
-      <c r="N75" t="n">
+      <c r="N75" s="18" t="n">
         <v>293</v>
       </c>
-      <c r="O75" t="inlineStr">
+      <c r="O75" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-05.csv</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="19">
-      <c r="A76" s="22" t="n"/>
+      <c r="A76" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>80</v>
+      </c>
+      <c r="C76" t="n">
+        <v>78</v>
+      </c>
+      <c r="D76" t="n">
+        <v>30488</v>
+      </c>
+      <c r="E76" t="n">
+        <v>259263</v>
+      </c>
+      <c r="F76" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="G76" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="H76" t="n">
+        <v>364</v>
+      </c>
+      <c r="I76" t="n">
+        <v>106</v>
+      </c>
+      <c r="J76" t="n">
+        <v>4610</v>
+      </c>
+      <c r="K76" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L76" t="n">
+        <v>26</v>
+      </c>
+      <c r="M76" t="n">
+        <v>195</v>
+      </c>
+      <c r="N76" t="n">
+        <v>294</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-06.csv</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="19">
       <c r="A77" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-07
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4367,53 +4367,101 @@
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="B76" t="n">
+      <c r="B76" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C76" t="n">
+      <c r="C76" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D76" t="n">
+      <c r="D76" s="18" t="n">
         <v>30488</v>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="18" t="n">
         <v>259263</v>
       </c>
-      <c r="F76" t="n">
+      <c r="F76" s="18" t="n">
         <v>11.54</v>
       </c>
-      <c r="G76" t="n">
+      <c r="G76" s="18" t="n">
         <v>48.5</v>
       </c>
-      <c r="H76" t="n">
+      <c r="H76" s="18" t="n">
         <v>364</v>
       </c>
-      <c r="I76" t="n">
+      <c r="I76" s="18" t="n">
         <v>106</v>
       </c>
-      <c r="J76" t="n">
+      <c r="J76" s="18" t="n">
         <v>4610</v>
       </c>
-      <c r="K76" t="n">
+      <c r="K76" s="18" t="n">
         <v>2.3</v>
       </c>
-      <c r="L76" t="n">
+      <c r="L76" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="M76" t="n">
+      <c r="M76" s="18" t="n">
         <v>195</v>
       </c>
-      <c r="N76" t="n">
+      <c r="N76" s="18" t="n">
         <v>294</v>
       </c>
-      <c r="O76" t="inlineStr">
+      <c r="O76" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-06.csv</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="19">
-      <c r="A77" s="22" t="n"/>
+      <c r="A77" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>80</v>
+      </c>
+      <c r="C77" t="n">
+        <v>78</v>
+      </c>
+      <c r="D77" t="n">
+        <v>30682</v>
+      </c>
+      <c r="E77" t="n">
+        <v>260501</v>
+      </c>
+      <c r="F77" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="G77" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="H77" t="n">
+        <v>366</v>
+      </c>
+      <c r="I77" t="n">
+        <v>107</v>
+      </c>
+      <c r="J77" t="n">
+        <v>4597</v>
+      </c>
+      <c r="K77" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="L77" t="n">
+        <v>26</v>
+      </c>
+      <c r="M77" t="n">
+        <v>200</v>
+      </c>
+      <c r="N77" t="n">
+        <v>295</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-07.csv</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="19">
       <c r="A78" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-08
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4418,53 +4418,101 @@
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B77" t="n">
+      <c r="B77" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C77" t="n">
+      <c r="C77" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D77" t="n">
+      <c r="D77" s="18" t="n">
         <v>30682</v>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="18" t="n">
         <v>260501</v>
       </c>
-      <c r="F77" t="n">
+      <c r="F77" s="18" t="n">
         <v>11.56</v>
       </c>
-      <c r="G77" t="n">
+      <c r="G77" s="18" t="n">
         <v>48.5</v>
       </c>
-      <c r="H77" t="n">
+      <c r="H77" s="18" t="n">
         <v>366</v>
       </c>
-      <c r="I77" t="n">
+      <c r="I77" s="18" t="n">
         <v>107</v>
       </c>
-      <c r="J77" t="n">
+      <c r="J77" s="18" t="n">
         <v>4597</v>
       </c>
-      <c r="K77" t="n">
+      <c r="K77" s="18" t="n">
         <v>2.33</v>
       </c>
-      <c r="L77" t="n">
+      <c r="L77" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="M77" t="n">
+      <c r="M77" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="N77" t="n">
+      <c r="N77" s="18" t="n">
         <v>295</v>
       </c>
-      <c r="O77" t="inlineStr">
+      <c r="O77" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-07.csv</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="19">
-      <c r="A78" s="22" t="n"/>
+      <c r="A78" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>80</v>
+      </c>
+      <c r="C78" t="n">
+        <v>78</v>
+      </c>
+      <c r="D78" t="n">
+        <v>30777</v>
+      </c>
+      <c r="E78" t="n">
+        <v>261161</v>
+      </c>
+      <c r="F78" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="G78" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="H78" t="n">
+        <v>374</v>
+      </c>
+      <c r="I78" t="n">
+        <v>107</v>
+      </c>
+      <c r="J78" t="n">
+        <v>4588</v>
+      </c>
+      <c r="K78" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="L78" t="n">
+        <v>27</v>
+      </c>
+      <c r="M78" t="n">
+        <v>205</v>
+      </c>
+      <c r="N78" t="n">
+        <v>299</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-08.csv</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="19">
       <c r="A79" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-09
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4469,53 +4469,101 @@
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="B78" t="n">
+      <c r="B78" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C78" t="n">
+      <c r="C78" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D78" t="n">
+      <c r="D78" s="18" t="n">
         <v>30777</v>
       </c>
-      <c r="E78" t="n">
+      <c r="E78" s="18" t="n">
         <v>261161</v>
       </c>
-      <c r="F78" t="n">
+      <c r="F78" s="18" t="n">
         <v>11.57</v>
       </c>
-      <c r="G78" t="n">
+      <c r="G78" s="18" t="n">
         <v>48.5</v>
       </c>
-      <c r="H78" t="n">
+      <c r="H78" s="18" t="n">
         <v>374</v>
       </c>
-      <c r="I78" t="n">
+      <c r="I78" s="18" t="n">
         <v>107</v>
       </c>
-      <c r="J78" t="n">
+      <c r="J78" s="18" t="n">
         <v>4588</v>
       </c>
-      <c r="K78" t="n">
+      <c r="K78" s="18" t="n">
         <v>2.33</v>
       </c>
-      <c r="L78" t="n">
+      <c r="L78" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="M78" t="n">
+      <c r="M78" s="18" t="n">
         <v>205</v>
       </c>
-      <c r="N78" t="n">
+      <c r="N78" s="18" t="n">
         <v>299</v>
       </c>
-      <c r="O78" t="inlineStr">
+      <c r="O78" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-08.csv</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="19">
-      <c r="A79" s="22" t="n"/>
+      <c r="A79" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>80</v>
+      </c>
+      <c r="C79" t="n">
+        <v>78</v>
+      </c>
+      <c r="D79" t="n">
+        <v>30792</v>
+      </c>
+      <c r="E79" t="n">
+        <v>261122</v>
+      </c>
+      <c r="F79" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="G79" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="H79" t="n">
+        <v>377</v>
+      </c>
+      <c r="I79" t="n">
+        <v>102</v>
+      </c>
+      <c r="J79" t="n">
+        <v>4508</v>
+      </c>
+      <c r="K79" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="L79" t="n">
+        <v>26</v>
+      </c>
+      <c r="M79" t="n">
+        <v>207</v>
+      </c>
+      <c r="N79" t="n">
+        <v>297</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-09.csv</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="19">
       <c r="A80" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-10
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4520,53 +4520,101 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B79" t="n">
+      <c r="B79" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D79" t="n">
+      <c r="D79" s="18" t="n">
         <v>30792</v>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="18" t="n">
         <v>261122</v>
       </c>
-      <c r="F79" t="n">
+      <c r="F79" s="18" t="n">
         <v>11.58</v>
       </c>
-      <c r="G79" t="n">
+      <c r="G79" s="18" t="n">
         <v>48.6</v>
       </c>
-      <c r="H79" t="n">
+      <c r="H79" s="18" t="n">
         <v>377</v>
       </c>
-      <c r="I79" t="n">
+      <c r="I79" s="18" t="n">
         <v>102</v>
       </c>
-      <c r="J79" t="n">
+      <c r="J79" s="18" t="n">
         <v>4508</v>
       </c>
-      <c r="K79" t="n">
+      <c r="K79" s="18" t="n">
         <v>2.26</v>
       </c>
-      <c r="L79" t="n">
+      <c r="L79" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="M79" t="n">
+      <c r="M79" s="18" t="n">
         <v>207</v>
       </c>
-      <c r="N79" t="n">
+      <c r="N79" s="18" t="n">
         <v>297</v>
       </c>
-      <c r="O79" t="inlineStr">
+      <c r="O79" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-09.csv</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="19">
-      <c r="A80" s="22" t="n"/>
+      <c r="A80" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>81</v>
+      </c>
+      <c r="C80" t="n">
+        <v>78</v>
+      </c>
+      <c r="D80" t="n">
+        <v>30888</v>
+      </c>
+      <c r="E80" t="n">
+        <v>262740</v>
+      </c>
+      <c r="F80" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="G80" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="H80" t="n">
+        <v>379</v>
+      </c>
+      <c r="I80" t="n">
+        <v>98</v>
+      </c>
+      <c r="J80" t="n">
+        <v>4440</v>
+      </c>
+      <c r="K80" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="L80" t="n">
+        <v>27</v>
+      </c>
+      <c r="M80" t="n">
+        <v>210</v>
+      </c>
+      <c r="N80" t="n">
+        <v>298</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-10.csv</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="19">
       <c r="A81" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-11
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4571,53 +4571,101 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B80" t="n">
+      <c r="B80" s="18" t="n">
         <v>81</v>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="D80" t="n">
+      <c r="D80" s="18" t="n">
         <v>30888</v>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="18" t="n">
         <v>262740</v>
       </c>
-      <c r="F80" t="n">
+      <c r="F80" s="18" t="n">
         <v>11.54</v>
       </c>
-      <c r="G80" t="n">
+      <c r="G80" s="18" t="n">
         <v>48.7</v>
       </c>
-      <c r="H80" t="n">
+      <c r="H80" s="18" t="n">
         <v>379</v>
       </c>
-      <c r="I80" t="n">
+      <c r="I80" s="18" t="n">
         <v>98</v>
       </c>
-      <c r="J80" t="n">
+      <c r="J80" s="18" t="n">
         <v>4440</v>
       </c>
-      <c r="K80" t="n">
+      <c r="K80" s="18" t="n">
         <v>2.21</v>
       </c>
-      <c r="L80" t="n">
+      <c r="L80" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="M80" t="n">
+      <c r="M80" s="18" t="n">
         <v>210</v>
       </c>
-      <c r="N80" t="n">
+      <c r="N80" s="18" t="n">
         <v>298</v>
       </c>
-      <c r="O80" t="inlineStr">
+      <c r="O80" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-10.csv</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="19">
-      <c r="A81" s="22" t="n"/>
+      <c r="A81" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>82</v>
+      </c>
+      <c r="C81" t="n">
+        <v>79</v>
+      </c>
+      <c r="D81" t="n">
+        <v>30892</v>
+      </c>
+      <c r="E81" t="n">
+        <v>263152</v>
+      </c>
+      <c r="F81" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="G81" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="H81" t="n">
+        <v>382</v>
+      </c>
+      <c r="I81" t="n">
+        <v>101</v>
+      </c>
+      <c r="J81" t="n">
+        <v>4416</v>
+      </c>
+      <c r="K81" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="L81" t="n">
+        <v>31</v>
+      </c>
+      <c r="M81" t="n">
+        <v>211</v>
+      </c>
+      <c r="N81" t="n">
+        <v>300</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-11.csv</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="19">
       <c r="A82" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-12
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4622,53 +4622,101 @@
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B81" t="n">
+      <c r="B81" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="D81" t="n">
+      <c r="D81" s="18" t="n">
         <v>30892</v>
       </c>
-      <c r="E81" t="n">
+      <c r="E81" s="18" t="n">
         <v>263152</v>
       </c>
-      <c r="F81" t="n">
+      <c r="F81" s="18" t="n">
         <v>11.52</v>
       </c>
-      <c r="G81" t="n">
+      <c r="G81" s="18" t="n">
         <v>48.5</v>
       </c>
-      <c r="H81" t="n">
+      <c r="H81" s="18" t="n">
         <v>382</v>
       </c>
-      <c r="I81" t="n">
+      <c r="I81" s="18" t="n">
         <v>101</v>
       </c>
-      <c r="J81" t="n">
+      <c r="J81" s="18" t="n">
         <v>4416</v>
       </c>
-      <c r="K81" t="n">
+      <c r="K81" s="18" t="n">
         <v>2.29</v>
       </c>
-      <c r="L81" t="n">
+      <c r="L81" s="18" t="n">
         <v>31</v>
       </c>
-      <c r="M81" t="n">
+      <c r="M81" s="18" t="n">
         <v>211</v>
       </c>
-      <c r="N81" t="n">
+      <c r="N81" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="O81" t="inlineStr">
+      <c r="O81" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-11.csv</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="19">
-      <c r="A82" s="22" t="n"/>
+      <c r="A82" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>82</v>
+      </c>
+      <c r="C82" t="n">
+        <v>79</v>
+      </c>
+      <c r="D82" t="n">
+        <v>36802</v>
+      </c>
+      <c r="E82" t="n">
+        <v>325525</v>
+      </c>
+      <c r="F82" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="G82" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="H82" t="n">
+        <v>384</v>
+      </c>
+      <c r="I82" t="n">
+        <v>101</v>
+      </c>
+      <c r="J82" t="n">
+        <v>4400</v>
+      </c>
+      <c r="K82" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L82" t="n">
+        <v>33</v>
+      </c>
+      <c r="M82" t="n">
+        <v>209</v>
+      </c>
+      <c r="N82" t="n">
+        <v>300</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-12.csv</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="19">
       <c r="A83" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-13
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4673,53 +4673,101 @@
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="B82" t="n">
+      <c r="B82" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="D82" t="n">
+      <c r="D82" s="18" t="n">
         <v>36802</v>
       </c>
-      <c r="E82" t="n">
+      <c r="E82" s="18" t="n">
         <v>325525</v>
       </c>
-      <c r="F82" t="n">
+      <c r="F82" s="18" t="n">
         <v>11.13</v>
       </c>
-      <c r="G82" t="n">
+      <c r="G82" s="18" t="n">
         <v>48.7</v>
       </c>
-      <c r="H82" t="n">
+      <c r="H82" s="18" t="n">
         <v>384</v>
       </c>
-      <c r="I82" t="n">
+      <c r="I82" s="18" t="n">
         <v>101</v>
       </c>
-      <c r="J82" t="n">
+      <c r="J82" s="18" t="n">
         <v>4400</v>
       </c>
-      <c r="K82" t="n">
+      <c r="K82" s="18" t="n">
         <v>2.3</v>
       </c>
-      <c r="L82" t="n">
+      <c r="L82" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="M82" t="n">
+      <c r="M82" s="18" t="n">
         <v>209</v>
       </c>
-      <c r="N82" t="n">
+      <c r="N82" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="O82" t="inlineStr">
+      <c r="O82" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-12.csv</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="19">
-      <c r="A83" s="22" t="n"/>
+      <c r="A83" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" t="n">
+        <v>80</v>
+      </c>
+      <c r="D83" t="n">
+        <v>42161</v>
+      </c>
+      <c r="E83" t="n">
+        <v>367215</v>
+      </c>
+      <c r="F83" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="G83" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H83" t="n">
+        <v>389</v>
+      </c>
+      <c r="I83" t="n">
+        <v>99</v>
+      </c>
+      <c r="J83" t="n">
+        <v>4361</v>
+      </c>
+      <c r="K83" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="L83" t="n">
+        <v>32</v>
+      </c>
+      <c r="M83" t="n">
+        <v>211</v>
+      </c>
+      <c r="N83" t="n">
+        <v>301</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-13.csv</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="19">
       <c r="A84" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-14
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4724,53 +4724,101 @@
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B83" t="n">
+      <c r="B83" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C83" t="n">
+      <c r="C83" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D83" t="n">
+      <c r="D83" s="18" t="n">
         <v>42161</v>
       </c>
-      <c r="E83" t="n">
+      <c r="E83" s="18" t="n">
         <v>367215</v>
       </c>
-      <c r="F83" t="n">
+      <c r="F83" s="18" t="n">
         <v>11.33</v>
       </c>
-      <c r="G83" t="n">
+      <c r="G83" s="18" t="n">
         <v>48.9</v>
       </c>
-      <c r="H83" t="n">
+      <c r="H83" s="18" t="n">
         <v>389</v>
       </c>
-      <c r="I83" t="n">
+      <c r="I83" s="18" t="n">
         <v>99</v>
       </c>
-      <c r="J83" t="n">
+      <c r="J83" s="18" t="n">
         <v>4361</v>
       </c>
-      <c r="K83" t="n">
+      <c r="K83" s="18" t="n">
         <v>2.27</v>
       </c>
-      <c r="L83" t="n">
+      <c r="L83" s="18" t="n">
         <v>32</v>
       </c>
-      <c r="M83" t="n">
+      <c r="M83" s="18" t="n">
         <v>211</v>
       </c>
-      <c r="N83" t="n">
+      <c r="N83" s="18" t="n">
         <v>301</v>
       </c>
-      <c r="O83" t="inlineStr">
+      <c r="O83" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-13.csv</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="19">
-      <c r="A84" s="22" t="n"/>
+      <c r="A84" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>82</v>
+      </c>
+      <c r="C84" t="n">
+        <v>80</v>
+      </c>
+      <c r="D84" t="n">
+        <v>44531</v>
+      </c>
+      <c r="E84" t="n">
+        <v>388674</v>
+      </c>
+      <c r="F84" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="G84" t="n">
+        <v>49</v>
+      </c>
+      <c r="H84" t="n">
+        <v>391</v>
+      </c>
+      <c r="I84" t="n">
+        <v>97</v>
+      </c>
+      <c r="J84" t="n">
+        <v>4305</v>
+      </c>
+      <c r="K84" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="L84" t="n">
+        <v>34</v>
+      </c>
+      <c r="M84" t="n">
+        <v>215</v>
+      </c>
+      <c r="N84" t="n">
+        <v>306</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-14.csv</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="19">
       <c r="A85" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-15
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4775,53 +4775,101 @@
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B84" t="n">
+      <c r="B84" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C84" t="n">
+      <c r="C84" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D84" t="n">
+      <c r="D84" s="18" t="n">
         <v>44531</v>
       </c>
-      <c r="E84" t="n">
+      <c r="E84" s="18" t="n">
         <v>388674</v>
       </c>
-      <c r="F84" t="n">
+      <c r="F84" s="18" t="n">
         <v>11.31</v>
       </c>
-      <c r="G84" t="n">
+      <c r="G84" s="18" t="n">
         <v>49</v>
       </c>
-      <c r="H84" t="n">
+      <c r="H84" s="18" t="n">
         <v>391</v>
       </c>
-      <c r="I84" t="n">
+      <c r="I84" s="18" t="n">
         <v>97</v>
       </c>
-      <c r="J84" t="n">
+      <c r="J84" s="18" t="n">
         <v>4305</v>
       </c>
-      <c r="K84" t="n">
+      <c r="K84" s="18" t="n">
         <v>2.25</v>
       </c>
-      <c r="L84" t="n">
+      <c r="L84" s="18" t="n">
         <v>34</v>
       </c>
-      <c r="M84" t="n">
+      <c r="M84" s="18" t="n">
         <v>215</v>
       </c>
-      <c r="N84" t="n">
+      <c r="N84" s="18" t="n">
         <v>306</v>
       </c>
-      <c r="O84" t="inlineStr">
+      <c r="O84" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-14.csv</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="19">
-      <c r="A85" s="22" t="n"/>
+      <c r="A85" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>82</v>
+      </c>
+      <c r="C85" t="n">
+        <v>80</v>
+      </c>
+      <c r="D85" t="n">
+        <v>45559</v>
+      </c>
+      <c r="E85" t="n">
+        <v>397177</v>
+      </c>
+      <c r="F85" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="G85" t="n">
+        <v>49</v>
+      </c>
+      <c r="H85" t="n">
+        <v>399</v>
+      </c>
+      <c r="I85" t="n">
+        <v>89</v>
+      </c>
+      <c r="J85" t="n">
+        <v>4339</v>
+      </c>
+      <c r="K85" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="L85" t="n">
+        <v>33</v>
+      </c>
+      <c r="M85" t="n">
+        <v>219</v>
+      </c>
+      <c r="N85" t="n">
+        <v>309</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-15.csv</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="19">
       <c r="A86" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-16
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4826,53 +4826,101 @@
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="B85" t="n">
+      <c r="B85" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D85" t="n">
+      <c r="D85" s="18" t="n">
         <v>45559</v>
       </c>
-      <c r="E85" t="n">
+      <c r="E85" s="18" t="n">
         <v>397177</v>
       </c>
-      <c r="F85" t="n">
+      <c r="F85" s="18" t="n">
         <v>11.33</v>
       </c>
-      <c r="G85" t="n">
+      <c r="G85" s="18" t="n">
         <v>49</v>
       </c>
-      <c r="H85" t="n">
+      <c r="H85" s="18" t="n">
         <v>399</v>
       </c>
-      <c r="I85" t="n">
+      <c r="I85" s="18" t="n">
         <v>89</v>
       </c>
-      <c r="J85" t="n">
+      <c r="J85" s="18" t="n">
         <v>4339</v>
       </c>
-      <c r="K85" t="n">
+      <c r="K85" s="18" t="n">
         <v>2.05</v>
       </c>
-      <c r="L85" t="n">
+      <c r="L85" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="M85" t="n">
+      <c r="M85" s="18" t="n">
         <v>219</v>
       </c>
-      <c r="N85" t="n">
+      <c r="N85" s="18" t="n">
         <v>309</v>
       </c>
-      <c r="O85" t="inlineStr">
+      <c r="O85" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-15.csv</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="19">
-      <c r="A86" s="22" t="n"/>
+      <c r="A86" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>82</v>
+      </c>
+      <c r="C86" t="n">
+        <v>80</v>
+      </c>
+      <c r="D86" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E86" t="n">
+        <v>405970</v>
+      </c>
+      <c r="F86" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="G86" t="n">
+        <v>49</v>
+      </c>
+      <c r="H86" t="n">
+        <v>401</v>
+      </c>
+      <c r="I86" t="n">
+        <v>84</v>
+      </c>
+      <c r="J86" t="n">
+        <v>4351</v>
+      </c>
+      <c r="K86" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="L86" t="n">
+        <v>33</v>
+      </c>
+      <c r="M86" t="n">
+        <v>216</v>
+      </c>
+      <c r="N86" t="n">
+        <v>309</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-16.csv</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="19">
       <c r="A87" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-17
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4877,53 +4877,101 @@
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="B86" t="n">
+      <c r="B86" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D86" t="n">
+      <c r="D86" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="E86" t="n">
+      <c r="E86" s="18" t="n">
         <v>405970</v>
       </c>
-      <c r="F86" t="n">
+      <c r="F86" s="18" t="n">
         <v>11.26</v>
       </c>
-      <c r="G86" t="n">
+      <c r="G86" s="18" t="n">
         <v>49</v>
       </c>
-      <c r="H86" t="n">
+      <c r="H86" s="18" t="n">
         <v>401</v>
       </c>
-      <c r="I86" t="n">
+      <c r="I86" s="18" t="n">
         <v>84</v>
       </c>
-      <c r="J86" t="n">
+      <c r="J86" s="18" t="n">
         <v>4351</v>
       </c>
-      <c r="K86" t="n">
+      <c r="K86" s="18" t="n">
         <v>1.93</v>
       </c>
-      <c r="L86" t="n">
+      <c r="L86" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="M86" t="n">
+      <c r="M86" s="18" t="n">
         <v>216</v>
       </c>
-      <c r="N86" t="n">
+      <c r="N86" s="18" t="n">
         <v>309</v>
       </c>
-      <c r="O86" t="inlineStr">
+      <c r="O86" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-16.csv</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="19">
-      <c r="A87" s="22" t="n"/>
+      <c r="A87" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>82</v>
+      </c>
+      <c r="C87" t="n">
+        <v>80</v>
+      </c>
+      <c r="D87" t="n">
+        <v>46816</v>
+      </c>
+      <c r="E87" t="n">
+        <v>411428</v>
+      </c>
+      <c r="F87" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="G87" t="n">
+        <v>49</v>
+      </c>
+      <c r="H87" t="n">
+        <v>406</v>
+      </c>
+      <c r="I87" t="n">
+        <v>82</v>
+      </c>
+      <c r="J87" t="n">
+        <v>4379</v>
+      </c>
+      <c r="K87" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="L87" t="n">
+        <v>32</v>
+      </c>
+      <c r="M87" t="n">
+        <v>223</v>
+      </c>
+      <c r="N87" t="n">
+        <v>315</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-17.csv</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="19">
       <c r="A88" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-18
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4928,53 +4928,101 @@
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="B87" t="n">
+      <c r="B87" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C87" t="n">
+      <c r="C87" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D87" t="n">
+      <c r="D87" s="18" t="n">
         <v>46816</v>
       </c>
-      <c r="E87" t="n">
+      <c r="E87" s="18" t="n">
         <v>411428</v>
       </c>
-      <c r="F87" t="n">
+      <c r="F87" s="18" t="n">
         <v>11.24</v>
       </c>
-      <c r="G87" t="n">
+      <c r="G87" s="18" t="n">
         <v>49</v>
       </c>
-      <c r="H87" t="n">
+      <c r="H87" s="18" t="n">
         <v>406</v>
       </c>
-      <c r="I87" t="n">
+      <c r="I87" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="J87" t="n">
+      <c r="J87" s="18" t="n">
         <v>4379</v>
       </c>
-      <c r="K87" t="n">
+      <c r="K87" s="18" t="n">
         <v>1.87</v>
       </c>
-      <c r="L87" t="n">
+      <c r="L87" s="18" t="n">
         <v>32</v>
       </c>
-      <c r="M87" t="n">
+      <c r="M87" s="18" t="n">
         <v>223</v>
       </c>
-      <c r="N87" t="n">
+      <c r="N87" s="18" t="n">
         <v>315</v>
       </c>
-      <c r="O87" t="inlineStr">
+      <c r="O87" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-17.csv</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="19">
-      <c r="A88" s="22" t="n"/>
+      <c r="A88" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>82</v>
+      </c>
+      <c r="C88" t="n">
+        <v>80</v>
+      </c>
+      <c r="D88" t="n">
+        <v>47307</v>
+      </c>
+      <c r="E88" t="n">
+        <v>415139</v>
+      </c>
+      <c r="F88" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="G88" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="H88" t="n">
+        <v>407</v>
+      </c>
+      <c r="I88" t="n">
+        <v>80</v>
+      </c>
+      <c r="J88" t="n">
+        <v>4334</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="L88" t="n">
+        <v>35</v>
+      </c>
+      <c r="M88" t="n">
+        <v>223</v>
+      </c>
+      <c r="N88" t="n">
+        <v>317</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-18.csv</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="19">
       <c r="A89" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-19
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -4979,53 +4979,101 @@
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="B88" t="n">
+      <c r="B88" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C88" t="n">
+      <c r="C88" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D88" t="n">
+      <c r="D88" s="18" t="n">
         <v>47307</v>
       </c>
-      <c r="E88" t="n">
+      <c r="E88" s="18" t="n">
         <v>415139</v>
       </c>
-      <c r="F88" t="n">
+      <c r="F88" s="18" t="n">
         <v>11.26</v>
       </c>
-      <c r="G88" t="n">
+      <c r="G88" s="18" t="n">
         <v>49.1</v>
       </c>
-      <c r="H88" t="n">
+      <c r="H88" s="18" t="n">
         <v>407</v>
       </c>
-      <c r="I88" t="n">
+      <c r="I88" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="J88" t="n">
+      <c r="J88" s="18" t="n">
         <v>4334</v>
       </c>
-      <c r="K88" t="n">
+      <c r="K88" s="18" t="n">
         <v>1.85</v>
       </c>
-      <c r="L88" t="n">
+      <c r="L88" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="M88" t="n">
+      <c r="M88" s="18" t="n">
         <v>223</v>
       </c>
-      <c r="N88" t="n">
+      <c r="N88" s="18" t="n">
         <v>317</v>
       </c>
-      <c r="O88" t="inlineStr">
+      <c r="O88" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-18.csv</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="19">
-      <c r="A89" s="22" t="n"/>
+      <c r="A89" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>82</v>
+      </c>
+      <c r="C89" t="n">
+        <v>80</v>
+      </c>
+      <c r="D89" t="n">
+        <v>45560</v>
+      </c>
+      <c r="E89" t="n">
+        <v>407144</v>
+      </c>
+      <c r="F89" t="n">
+        <v>11.05</v>
+      </c>
+      <c r="G89" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H89" t="n">
+        <v>412</v>
+      </c>
+      <c r="I89" t="n">
+        <v>73</v>
+      </c>
+      <c r="J89" t="n">
+        <v>4279</v>
+      </c>
+      <c r="K89" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="L89" t="n">
+        <v>35</v>
+      </c>
+      <c r="M89" t="n">
+        <v>229</v>
+      </c>
+      <c r="N89" t="n">
+        <v>323</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-19.csv</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="19">
       <c r="A90" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-20
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5030,53 +5030,101 @@
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="B89" t="n">
+      <c r="B89" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C89" t="n">
+      <c r="C89" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D89" t="n">
+      <c r="D89" s="18" t="n">
         <v>45560</v>
       </c>
-      <c r="E89" t="n">
+      <c r="E89" s="18" t="n">
         <v>407144</v>
       </c>
-      <c r="F89" t="n">
+      <c r="F89" s="18" t="n">
         <v>11.05</v>
       </c>
-      <c r="G89" t="n">
+      <c r="G89" s="18" t="n">
         <v>48.9</v>
       </c>
-      <c r="H89" t="n">
+      <c r="H89" s="18" t="n">
         <v>412</v>
       </c>
-      <c r="I89" t="n">
+      <c r="I89" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="J89" t="n">
+      <c r="J89" s="18" t="n">
         <v>4279</v>
       </c>
-      <c r="K89" t="n">
+      <c r="K89" s="18" t="n">
         <v>1.71</v>
       </c>
-      <c r="L89" t="n">
+      <c r="L89" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="M89" t="n">
+      <c r="M89" s="18" t="n">
         <v>229</v>
       </c>
-      <c r="N89" t="n">
+      <c r="N89" s="18" t="n">
         <v>323</v>
       </c>
-      <c r="O89" t="inlineStr">
+      <c r="O89" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-19.csv</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="19">
-      <c r="A90" s="22" t="n"/>
+      <c r="A90" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>82</v>
+      </c>
+      <c r="C90" t="n">
+        <v>80</v>
+      </c>
+      <c r="D90" t="n">
+        <v>44804</v>
+      </c>
+      <c r="E90" t="n">
+        <v>402982</v>
+      </c>
+      <c r="F90" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="G90" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="H90" t="n">
+        <v>413</v>
+      </c>
+      <c r="I90" t="n">
+        <v>72</v>
+      </c>
+      <c r="J90" t="n">
+        <v>4282</v>
+      </c>
+      <c r="K90" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="L90" t="n">
+        <v>35</v>
+      </c>
+      <c r="M90" t="n">
+        <v>221</v>
+      </c>
+      <c r="N90" t="n">
+        <v>323</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-20.csv</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="19">
       <c r="A91" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-21
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5081,53 +5081,101 @@
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B90" t="n">
+      <c r="B90" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C90" t="n">
+      <c r="C90" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D90" t="n">
+      <c r="D90" s="18" t="n">
         <v>44804</v>
       </c>
-      <c r="E90" t="n">
+      <c r="E90" s="18" t="n">
         <v>402982</v>
       </c>
-      <c r="F90" t="n">
+      <c r="F90" s="18" t="n">
         <v>10.98</v>
       </c>
-      <c r="G90" t="n">
+      <c r="G90" s="18" t="n">
         <v>48.8</v>
       </c>
-      <c r="H90" t="n">
+      <c r="H90" s="18" t="n">
         <v>413</v>
       </c>
-      <c r="I90" t="n">
+      <c r="I90" s="18" t="n">
         <v>72</v>
       </c>
-      <c r="J90" t="n">
+      <c r="J90" s="18" t="n">
         <v>4282</v>
       </c>
-      <c r="K90" t="n">
+      <c r="K90" s="18" t="n">
         <v>1.68</v>
       </c>
-      <c r="L90" t="n">
+      <c r="L90" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="M90" t="n">
+      <c r="M90" s="18" t="n">
         <v>221</v>
       </c>
-      <c r="N90" t="n">
+      <c r="N90" s="18" t="n">
         <v>323</v>
       </c>
-      <c r="O90" t="inlineStr">
+      <c r="O90" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-20.csv</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="19">
-      <c r="A91" s="22" t="n"/>
+      <c r="A91" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>82</v>
+      </c>
+      <c r="C91" t="n">
+        <v>80</v>
+      </c>
+      <c r="D91" t="n">
+        <v>44477</v>
+      </c>
+      <c r="E91" t="n">
+        <v>401159</v>
+      </c>
+      <c r="F91" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="G91" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="H91" t="n">
+        <v>412</v>
+      </c>
+      <c r="I91" t="n">
+        <v>73</v>
+      </c>
+      <c r="J91" t="n">
+        <v>4285</v>
+      </c>
+      <c r="K91" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L91" t="n">
+        <v>37</v>
+      </c>
+      <c r="M91" t="n">
+        <v>219</v>
+      </c>
+      <c r="N91" t="n">
+        <v>322</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-21.csv</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="19">
       <c r="A92" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-22
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5132,53 +5132,101 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B91" t="n">
+      <c r="B91" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C91" t="n">
+      <c r="C91" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D91" t="n">
+      <c r="D91" s="18" t="n">
         <v>44477</v>
       </c>
-      <c r="E91" t="n">
+      <c r="E91" s="18" t="n">
         <v>401159</v>
       </c>
-      <c r="F91" t="n">
+      <c r="F91" s="18" t="n">
         <v>10.95</v>
       </c>
-      <c r="G91" t="n">
+      <c r="G91" s="18" t="n">
         <v>48.8</v>
       </c>
-      <c r="H91" t="n">
+      <c r="H91" s="18" t="n">
         <v>412</v>
       </c>
-      <c r="I91" t="n">
+      <c r="I91" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="J91" t="n">
+      <c r="J91" s="18" t="n">
         <v>4285</v>
       </c>
-      <c r="K91" t="n">
+      <c r="K91" s="18" t="n">
         <v>1.7</v>
       </c>
-      <c r="L91" t="n">
+      <c r="L91" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="M91" t="n">
+      <c r="M91" s="18" t="n">
         <v>219</v>
       </c>
-      <c r="N91" t="n">
+      <c r="N91" s="18" t="n">
         <v>322</v>
       </c>
-      <c r="O91" t="inlineStr">
+      <c r="O91" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-21.csv</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="19">
-      <c r="A92" s="22" t="n"/>
+      <c r="A92" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>82</v>
+      </c>
+      <c r="C92" t="n">
+        <v>80</v>
+      </c>
+      <c r="D92" t="n">
+        <v>44446</v>
+      </c>
+      <c r="E92" t="n">
+        <v>400615</v>
+      </c>
+      <c r="F92" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="G92" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="H92" t="n">
+        <v>410</v>
+      </c>
+      <c r="I92" t="n">
+        <v>70</v>
+      </c>
+      <c r="J92" t="n">
+        <v>4250</v>
+      </c>
+      <c r="K92" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="L92" t="n">
+        <v>36</v>
+      </c>
+      <c r="M92" t="n">
+        <v>219</v>
+      </c>
+      <c r="N92" t="n">
+        <v>318</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-22.csv</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="19">
       <c r="A93" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-23
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5183,53 +5183,101 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B92" t="n">
+      <c r="B92" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C92" t="n">
+      <c r="C92" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D92" t="n">
+      <c r="D92" s="18" t="n">
         <v>44446</v>
       </c>
-      <c r="E92" t="n">
+      <c r="E92" s="18" t="n">
         <v>400615</v>
       </c>
-      <c r="F92" t="n">
+      <c r="F92" s="18" t="n">
         <v>10.96</v>
       </c>
-      <c r="G92" t="n">
+      <c r="G92" s="18" t="n">
         <v>48.7</v>
       </c>
-      <c r="H92" t="n">
+      <c r="H92" s="18" t="n">
         <v>410</v>
       </c>
-      <c r="I92" t="n">
+      <c r="I92" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="J92" t="n">
+      <c r="J92" s="18" t="n">
         <v>4250</v>
       </c>
-      <c r="K92" t="n">
+      <c r="K92" s="18" t="n">
         <v>1.65</v>
       </c>
-      <c r="L92" t="n">
+      <c r="L92" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="M92" t="n">
+      <c r="M92" s="18" t="n">
         <v>219</v>
       </c>
-      <c r="N92" t="n">
+      <c r="N92" s="18" t="n">
         <v>318</v>
       </c>
-      <c r="O92" t="inlineStr">
+      <c r="O92" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-22.csv</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="19">
-      <c r="A93" s="22" t="n"/>
+      <c r="A93" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>82</v>
+      </c>
+      <c r="C93" t="n">
+        <v>80</v>
+      </c>
+      <c r="D93" t="n">
+        <v>42248</v>
+      </c>
+      <c r="E93" t="n">
+        <v>389229</v>
+      </c>
+      <c r="F93" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="G93" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="H93" t="n">
+        <v>426</v>
+      </c>
+      <c r="I93" t="n">
+        <v>69</v>
+      </c>
+      <c r="J93" t="n">
+        <v>4252</v>
+      </c>
+      <c r="K93" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="L93" t="n">
+        <v>40</v>
+      </c>
+      <c r="M93" t="n">
+        <v>222</v>
+      </c>
+      <c r="N93" t="n">
+        <v>325</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-23.csv</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="19">
       <c r="A94" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-24
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5234,53 +5234,101 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B93" t="n">
+      <c r="B93" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C93" t="n">
+      <c r="C93" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D93" t="n">
+      <c r="D93" s="18" t="n">
         <v>42248</v>
       </c>
-      <c r="E93" t="n">
+      <c r="E93" s="18" t="n">
         <v>389229</v>
       </c>
-      <c r="F93" t="n">
+      <c r="F93" s="18" t="n">
         <v>10.71</v>
       </c>
-      <c r="G93" t="n">
+      <c r="G93" s="18" t="n">
         <v>48.7</v>
       </c>
-      <c r="H93" t="n">
+      <c r="H93" s="18" t="n">
         <v>426</v>
       </c>
-      <c r="I93" t="n">
+      <c r="I93" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="J93" t="n">
+      <c r="J93" s="18" t="n">
         <v>4252</v>
       </c>
-      <c r="K93" t="n">
+      <c r="K93" s="18" t="n">
         <v>1.62</v>
       </c>
-      <c r="L93" t="n">
+      <c r="L93" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M93" t="n">
+      <c r="M93" s="18" t="n">
         <v>222</v>
       </c>
-      <c r="N93" t="n">
+      <c r="N93" s="18" t="n">
         <v>325</v>
       </c>
-      <c r="O93" t="inlineStr">
+      <c r="O93" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-23.csv</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="19">
-      <c r="A94" s="22" t="n"/>
+      <c r="A94" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>82</v>
+      </c>
+      <c r="C94" t="n">
+        <v>80</v>
+      </c>
+      <c r="D94" t="n">
+        <v>39599</v>
+      </c>
+      <c r="E94" t="n">
+        <v>373380</v>
+      </c>
+      <c r="F94" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="G94" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="H94" t="n">
+        <v>433</v>
+      </c>
+      <c r="I94" t="n">
+        <v>68</v>
+      </c>
+      <c r="J94" t="n">
+        <v>4267</v>
+      </c>
+      <c r="K94" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="L94" t="n">
+        <v>40</v>
+      </c>
+      <c r="M94" t="n">
+        <v>219</v>
+      </c>
+      <c r="N94" t="n">
+        <v>324</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-24.csv</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="19">
       <c r="A95" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-25
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5285,53 +5285,101 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B94" t="n">
+      <c r="B94" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C94" t="n">
+      <c r="C94" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D94" t="n">
+      <c r="D94" s="18" t="n">
         <v>39599</v>
       </c>
-      <c r="E94" t="n">
+      <c r="E94" s="18" t="n">
         <v>373380</v>
       </c>
-      <c r="F94" t="n">
+      <c r="F94" s="18" t="n">
         <v>10.46</v>
       </c>
-      <c r="G94" t="n">
+      <c r="G94" s="18" t="n">
         <v>48.7</v>
       </c>
-      <c r="H94" t="n">
+      <c r="H94" s="18" t="n">
         <v>433</v>
       </c>
-      <c r="I94" t="n">
+      <c r="I94" s="18" t="n">
         <v>68</v>
       </c>
-      <c r="J94" t="n">
+      <c r="J94" s="18" t="n">
         <v>4267</v>
       </c>
-      <c r="K94" t="n">
+      <c r="K94" s="18" t="n">
         <v>1.59</v>
       </c>
-      <c r="L94" t="n">
+      <c r="L94" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M94" t="n">
+      <c r="M94" s="18" t="n">
         <v>219</v>
       </c>
-      <c r="N94" t="n">
+      <c r="N94" s="18" t="n">
         <v>324</v>
       </c>
-      <c r="O94" t="inlineStr">
+      <c r="O94" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-24.csv</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="19">
-      <c r="A95" s="22" t="n"/>
+      <c r="A95" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>82</v>
+      </c>
+      <c r="C95" t="n">
+        <v>80</v>
+      </c>
+      <c r="D95" t="n">
+        <v>37050</v>
+      </c>
+      <c r="E95" t="n">
+        <v>357872</v>
+      </c>
+      <c r="F95" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G95" t="n">
+        <v>49</v>
+      </c>
+      <c r="H95" t="n">
+        <v>428</v>
+      </c>
+      <c r="I95" t="n">
+        <v>68</v>
+      </c>
+      <c r="J95" t="n">
+        <v>4231</v>
+      </c>
+      <c r="K95" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="L95" t="n">
+        <v>40</v>
+      </c>
+      <c r="M95" t="n">
+        <v>218</v>
+      </c>
+      <c r="N95" t="n">
+        <v>321</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-25.csv</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="19">
       <c r="A96" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-26
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5336,53 +5336,101 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B95" t="n">
+      <c r="B95" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C95" t="n">
+      <c r="C95" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D95" t="n">
+      <c r="D95" s="18" t="n">
         <v>37050</v>
       </c>
-      <c r="E95" t="n">
+      <c r="E95" s="18" t="n">
         <v>357872</v>
       </c>
-      <c r="F95" t="n">
+      <c r="F95" s="18" t="n">
         <v>10.2</v>
       </c>
-      <c r="G95" t="n">
+      <c r="G95" s="18" t="n">
         <v>49</v>
       </c>
-      <c r="H95" t="n">
+      <c r="H95" s="18" t="n">
         <v>428</v>
       </c>
-      <c r="I95" t="n">
+      <c r="I95" s="18" t="n">
         <v>68</v>
       </c>
-      <c r="J95" t="n">
+      <c r="J95" s="18" t="n">
         <v>4231</v>
       </c>
-      <c r="K95" t="n">
+      <c r="K95" s="18" t="n">
         <v>1.61</v>
       </c>
-      <c r="L95" t="n">
+      <c r="L95" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M95" t="n">
+      <c r="M95" s="18" t="n">
         <v>218</v>
       </c>
-      <c r="N95" t="n">
+      <c r="N95" s="18" t="n">
         <v>321</v>
       </c>
-      <c r="O95" t="inlineStr">
+      <c r="O95" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-25.csv</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="19">
-      <c r="A96" s="22" t="n"/>
+      <c r="A96" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>82</v>
+      </c>
+      <c r="C96" t="n">
+        <v>80</v>
+      </c>
+      <c r="D96" t="n">
+        <v>35334</v>
+      </c>
+      <c r="E96" t="n">
+        <v>347089</v>
+      </c>
+      <c r="F96" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="G96" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="H96" t="n">
+        <v>429</v>
+      </c>
+      <c r="I96" t="n">
+        <v>69</v>
+      </c>
+      <c r="J96" t="n">
+        <v>4154</v>
+      </c>
+      <c r="K96" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="L96" t="n">
+        <v>40</v>
+      </c>
+      <c r="M96" t="n">
+        <v>217</v>
+      </c>
+      <c r="N96" t="n">
+        <v>319</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-26.csv</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="19">
       <c r="A97" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-27
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5387,53 +5387,101 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B96" t="n">
+      <c r="B96" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C96" t="n">
+      <c r="C96" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D96" t="n">
+      <c r="D96" s="18" t="n">
         <v>35334</v>
       </c>
-      <c r="E96" t="n">
+      <c r="E96" s="18" t="n">
         <v>347089</v>
       </c>
-      <c r="F96" t="n">
+      <c r="F96" s="18" t="n">
         <v>10.02</v>
       </c>
-      <c r="G96" t="n">
+      <c r="G96" s="18" t="n">
         <v>49.2</v>
       </c>
-      <c r="H96" t="n">
+      <c r="H96" s="18" t="n">
         <v>429</v>
       </c>
-      <c r="I96" t="n">
+      <c r="I96" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="J96" t="n">
+      <c r="J96" s="18" t="n">
         <v>4154</v>
       </c>
-      <c r="K96" t="n">
+      <c r="K96" s="18" t="n">
         <v>1.66</v>
       </c>
-      <c r="L96" t="n">
+      <c r="L96" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M96" t="n">
+      <c r="M96" s="18" t="n">
         <v>217</v>
       </c>
-      <c r="N96" t="n">
+      <c r="N96" s="18" t="n">
         <v>319</v>
       </c>
-      <c r="O96" t="inlineStr">
+      <c r="O96" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-26.csv</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="19">
-      <c r="A97" s="22" t="n"/>
+      <c r="A97" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>82</v>
+      </c>
+      <c r="C97" t="n">
+        <v>80</v>
+      </c>
+      <c r="D97" t="n">
+        <v>34167</v>
+      </c>
+      <c r="E97" t="n">
+        <v>339436</v>
+      </c>
+      <c r="F97" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G97" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="H97" t="n">
+        <v>434</v>
+      </c>
+      <c r="I97" t="n">
+        <v>73</v>
+      </c>
+      <c r="J97" t="n">
+        <v>4169</v>
+      </c>
+      <c r="K97" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="L97" t="n">
+        <v>39</v>
+      </c>
+      <c r="M97" t="n">
+        <v>220</v>
+      </c>
+      <c r="N97" t="n">
+        <v>320</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-27.csv</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="19">
       <c r="A98" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-28
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5438,53 +5438,101 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B97" t="n">
+      <c r="B97" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="C97" t="n">
+      <c r="C97" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D97" t="n">
+      <c r="D97" s="18" t="n">
         <v>34167</v>
       </c>
-      <c r="E97" t="n">
+      <c r="E97" s="18" t="n">
         <v>339436</v>
       </c>
-      <c r="F97" t="n">
+      <c r="F97" s="18" t="n">
         <v>9.9</v>
       </c>
-      <c r="G97" t="n">
+      <c r="G97" s="18" t="n">
         <v>47.9</v>
       </c>
-      <c r="H97" t="n">
+      <c r="H97" s="18" t="n">
         <v>434</v>
       </c>
-      <c r="I97" t="n">
+      <c r="I97" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="J97" t="n">
+      <c r="J97" s="18" t="n">
         <v>4169</v>
       </c>
-      <c r="K97" t="n">
+      <c r="K97" s="18" t="n">
         <v>1.75</v>
       </c>
-      <c r="L97" t="n">
+      <c r="L97" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="M97" t="n">
+      <c r="M97" s="18" t="n">
         <v>220</v>
       </c>
-      <c r="N97" t="n">
+      <c r="N97" s="18" t="n">
         <v>320</v>
       </c>
-      <c r="O97" t="inlineStr">
+      <c r="O97" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-27.csv</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="19">
-      <c r="A98" s="22" t="n"/>
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>83</v>
+      </c>
+      <c r="C98" t="n">
+        <v>80</v>
+      </c>
+      <c r="D98" t="n">
+        <v>33498</v>
+      </c>
+      <c r="E98" t="n">
+        <v>336336</v>
+      </c>
+      <c r="F98" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="G98" t="n">
+        <v>48</v>
+      </c>
+      <c r="H98" t="n">
+        <v>445</v>
+      </c>
+      <c r="I98" t="n">
+        <v>78</v>
+      </c>
+      <c r="J98" t="n">
+        <v>4169</v>
+      </c>
+      <c r="K98" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="L98" t="n">
+        <v>40</v>
+      </c>
+      <c r="M98" t="n">
+        <v>222</v>
+      </c>
+      <c r="N98" t="n">
+        <v>325</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-28.csv</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="19">
       <c r="A99" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-29
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5489,53 +5489,101 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B98" t="n">
+      <c r="B98" s="18" t="n">
         <v>83</v>
       </c>
-      <c r="C98" t="n">
+      <c r="C98" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D98" t="n">
+      <c r="D98" s="18" t="n">
         <v>33498</v>
       </c>
-      <c r="E98" t="n">
+      <c r="E98" s="18" t="n">
         <v>336336</v>
       </c>
-      <c r="F98" t="n">
+      <c r="F98" s="18" t="n">
         <v>9.789999999999999</v>
       </c>
-      <c r="G98" t="n">
+      <c r="G98" s="18" t="n">
         <v>48</v>
       </c>
-      <c r="H98" t="n">
+      <c r="H98" s="18" t="n">
         <v>445</v>
       </c>
-      <c r="I98" t="n">
+      <c r="I98" s="18" t="n">
         <v>78</v>
       </c>
-      <c r="J98" t="n">
+      <c r="J98" s="18" t="n">
         <v>4169</v>
       </c>
-      <c r="K98" t="n">
+      <c r="K98" s="18" t="n">
         <v>1.87</v>
       </c>
-      <c r="L98" t="n">
+      <c r="L98" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M98" t="n">
+      <c r="M98" s="18" t="n">
         <v>222</v>
       </c>
-      <c r="N98" t="n">
+      <c r="N98" s="18" t="n">
         <v>325</v>
       </c>
-      <c r="O98" t="inlineStr">
+      <c r="O98" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-28.csv</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="19">
-      <c r="A99" s="22" t="n"/>
+      <c r="A99" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>84</v>
+      </c>
+      <c r="C99" t="n">
+        <v>80</v>
+      </c>
+      <c r="D99" t="n">
+        <v>32879</v>
+      </c>
+      <c r="E99" t="n">
+        <v>332048</v>
+      </c>
+      <c r="F99" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="G99" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H99" t="n">
+        <v>447</v>
+      </c>
+      <c r="I99" t="n">
+        <v>75</v>
+      </c>
+      <c r="J99" t="n">
+        <v>4181</v>
+      </c>
+      <c r="K99" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="L99" t="n">
+        <v>40</v>
+      </c>
+      <c r="M99" t="n">
+        <v>227</v>
+      </c>
+      <c r="N99" t="n">
+        <v>329</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-29.csv</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="19">
       <c r="A100" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-30
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5540,53 +5540,101 @@
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B99" t="n">
+      <c r="B99" s="18" t="n">
         <v>84</v>
       </c>
-      <c r="C99" t="n">
+      <c r="C99" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D99" t="n">
+      <c r="D99" s="18" t="n">
         <v>32879</v>
       </c>
-      <c r="E99" t="n">
+      <c r="E99" s="18" t="n">
         <v>332048</v>
       </c>
-      <c r="F99" t="n">
+      <c r="F99" s="18" t="n">
         <v>9.73</v>
       </c>
-      <c r="G99" t="n">
+      <c r="G99" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H99" t="n">
+      <c r="H99" s="18" t="n">
         <v>447</v>
       </c>
-      <c r="I99" t="n">
+      <c r="I99" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="J99" t="n">
+      <c r="J99" s="18" t="n">
         <v>4181</v>
       </c>
-      <c r="K99" t="n">
+      <c r="K99" s="18" t="n">
         <v>1.79</v>
       </c>
-      <c r="L99" t="n">
+      <c r="L99" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M99" t="n">
+      <c r="M99" s="18" t="n">
         <v>227</v>
       </c>
-      <c r="N99" t="n">
+      <c r="N99" s="18" t="n">
         <v>329</v>
       </c>
-      <c r="O99" t="inlineStr">
+      <c r="O99" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-29.csv</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="19">
-      <c r="A100" s="22" t="n"/>
+      <c r="A100" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>84</v>
+      </c>
+      <c r="C100" t="n">
+        <v>80</v>
+      </c>
+      <c r="D100" t="n">
+        <v>32512</v>
+      </c>
+      <c r="E100" t="n">
+        <v>330878</v>
+      </c>
+      <c r="F100" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="G100" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="H100" t="n">
+        <v>448</v>
+      </c>
+      <c r="I100" t="n">
+        <v>74</v>
+      </c>
+      <c r="J100" t="n">
+        <v>4193</v>
+      </c>
+      <c r="K100" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="L100" t="n">
+        <v>41</v>
+      </c>
+      <c r="M100" t="n">
+        <v>224</v>
+      </c>
+      <c r="N100" t="n">
+        <v>327</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-30.csv</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="19">
       <c r="A101" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-08-31
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5591,53 +5591,101 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B100" t="n">
+      <c r="B100" s="18" t="n">
         <v>84</v>
       </c>
-      <c r="C100" t="n">
+      <c r="C100" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D100" t="n">
+      <c r="D100" s="18" t="n">
         <v>32512</v>
       </c>
-      <c r="E100" t="n">
+      <c r="E100" s="18" t="n">
         <v>330878</v>
       </c>
-      <c r="F100" t="n">
+      <c r="F100" s="18" t="n">
         <v>9.66</v>
       </c>
-      <c r="G100" t="n">
+      <c r="G100" s="18" t="n">
         <v>48.3</v>
       </c>
-      <c r="H100" t="n">
+      <c r="H100" s="18" t="n">
         <v>448</v>
       </c>
-      <c r="I100" t="n">
+      <c r="I100" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="J100" t="n">
+      <c r="J100" s="18" t="n">
         <v>4193</v>
       </c>
-      <c r="K100" t="n">
+      <c r="K100" s="18" t="n">
         <v>1.76</v>
       </c>
-      <c r="L100" t="n">
+      <c r="L100" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="M100" t="n">
+      <c r="M100" s="18" t="n">
         <v>224</v>
       </c>
-      <c r="N100" t="n">
+      <c r="N100" s="18" t="n">
         <v>327</v>
       </c>
-      <c r="O100" t="inlineStr">
+      <c r="O100" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-30.csv</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="19">
-      <c r="A101" s="22" t="n"/>
+      <c r="A101" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>85</v>
+      </c>
+      <c r="C101" t="n">
+        <v>82</v>
+      </c>
+      <c r="D101" t="n">
+        <v>36361</v>
+      </c>
+      <c r="E101" t="n">
+        <v>365639</v>
+      </c>
+      <c r="F101" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="G101" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H101" t="n">
+        <v>446</v>
+      </c>
+      <c r="I101" t="n">
+        <v>72</v>
+      </c>
+      <c r="J101" t="n">
+        <v>4128</v>
+      </c>
+      <c r="K101" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="L101" t="n">
+        <v>41</v>
+      </c>
+      <c r="M101" t="n">
+        <v>226</v>
+      </c>
+      <c r="N101" t="n">
+        <v>326</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-08-31.csv</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="19">
       <c r="A102" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-01
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5642,53 +5642,101 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B101" t="n">
+      <c r="B101" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="C101" t="n">
+      <c r="C101" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="D101" t="n">
+      <c r="D101" s="18" t="n">
         <v>36361</v>
       </c>
-      <c r="E101" t="n">
+      <c r="E101" s="18" t="n">
         <v>365639</v>
       </c>
-      <c r="F101" t="n">
+      <c r="F101" s="18" t="n">
         <v>9.789999999999999</v>
       </c>
-      <c r="G101" t="n">
+      <c r="G101" s="18" t="n">
         <v>48.2</v>
       </c>
-      <c r="H101" t="n">
+      <c r="H101" s="18" t="n">
         <v>446</v>
       </c>
-      <c r="I101" t="n">
+      <c r="I101" s="18" t="n">
         <v>72</v>
       </c>
-      <c r="J101" t="n">
+      <c r="J101" s="18" t="n">
         <v>4128</v>
       </c>
-      <c r="K101" t="n">
+      <c r="K101" s="18" t="n">
         <v>1.74</v>
       </c>
-      <c r="L101" t="n">
+      <c r="L101" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="M101" t="n">
+      <c r="M101" s="18" t="n">
         <v>226</v>
       </c>
-      <c r="N101" t="n">
+      <c r="N101" s="18" t="n">
         <v>326</v>
       </c>
-      <c r="O101" t="inlineStr">
+      <c r="O101" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-08-31.csv</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="19">
-      <c r="A102" s="22" t="n"/>
+      <c r="A102" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>93</v>
+      </c>
+      <c r="C102" t="n">
+        <v>82</v>
+      </c>
+      <c r="D102" t="n">
+        <v>42379</v>
+      </c>
+      <c r="E102" t="n">
+        <v>418578</v>
+      </c>
+      <c r="F102" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="G102" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H102" t="n">
+        <v>448</v>
+      </c>
+      <c r="I102" t="n">
+        <v>71</v>
+      </c>
+      <c r="J102" t="n">
+        <v>4076</v>
+      </c>
+      <c r="K102" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="L102" t="n">
+        <v>43</v>
+      </c>
+      <c r="M102" t="n">
+        <v>232</v>
+      </c>
+      <c r="N102" t="n">
+        <v>328</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-01.csv</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="19">
       <c r="A103" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-02
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5693,53 +5693,101 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B102" t="n">
+      <c r="B102" s="18" t="n">
         <v>93</v>
       </c>
-      <c r="C102" t="n">
+      <c r="C102" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="D102" t="n">
+      <c r="D102" s="18" t="n">
         <v>42379</v>
       </c>
-      <c r="E102" t="n">
+      <c r="E102" s="18" t="n">
         <v>418578</v>
       </c>
-      <c r="F102" t="n">
+      <c r="F102" s="18" t="n">
         <v>9.99</v>
       </c>
-      <c r="G102" t="n">
+      <c r="G102" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H102" t="n">
+      <c r="H102" s="18" t="n">
         <v>448</v>
       </c>
-      <c r="I102" t="n">
+      <c r="I102" s="18" t="n">
         <v>71</v>
       </c>
-      <c r="J102" t="n">
+      <c r="J102" s="18" t="n">
         <v>4076</v>
       </c>
-      <c r="K102" t="n">
+      <c r="K102" s="18" t="n">
         <v>1.74</v>
       </c>
-      <c r="L102" t="n">
+      <c r="L102" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="M102" t="n">
+      <c r="M102" s="18" t="n">
         <v>232</v>
       </c>
-      <c r="N102" t="n">
+      <c r="N102" s="18" t="n">
         <v>328</v>
       </c>
-      <c r="O102" t="inlineStr">
+      <c r="O102" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-01.csv</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="19">
-      <c r="A103" s="22" t="n"/>
+      <c r="A103" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>96</v>
+      </c>
+      <c r="C103" t="n">
+        <v>83</v>
+      </c>
+      <c r="D103" t="n">
+        <v>49443</v>
+      </c>
+      <c r="E103" t="n">
+        <v>476387</v>
+      </c>
+      <c r="F103" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="G103" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="H103" t="n">
+        <v>449</v>
+      </c>
+      <c r="I103" t="n">
+        <v>70</v>
+      </c>
+      <c r="J103" t="n">
+        <v>4061</v>
+      </c>
+      <c r="K103" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="L103" t="n">
+        <v>44</v>
+      </c>
+      <c r="M103" t="n">
+        <v>233</v>
+      </c>
+      <c r="N103" t="n">
+        <v>327</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-02.csv</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="19">
       <c r="A104" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-03
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5744,53 +5744,101 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B103" t="n">
+      <c r="B103" s="18" t="n">
         <v>96</v>
       </c>
-      <c r="C103" t="n">
+      <c r="C103" s="18" t="n">
         <v>83</v>
       </c>
-      <c r="D103" t="n">
+      <c r="D103" s="18" t="n">
         <v>49443</v>
       </c>
-      <c r="E103" t="n">
+      <c r="E103" s="18" t="n">
         <v>476387</v>
       </c>
-      <c r="F103" t="n">
+      <c r="F103" s="18" t="n">
         <v>10.26</v>
       </c>
-      <c r="G103" t="n">
+      <c r="G103" s="18" t="n">
         <v>48.1</v>
       </c>
-      <c r="H103" t="n">
+      <c r="H103" s="18" t="n">
         <v>449</v>
       </c>
-      <c r="I103" t="n">
+      <c r="I103" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="J103" t="n">
+      <c r="J103" s="18" t="n">
         <v>4061</v>
       </c>
-      <c r="K103" t="n">
+      <c r="K103" s="18" t="n">
         <v>1.72</v>
       </c>
-      <c r="L103" t="n">
+      <c r="L103" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="M103" t="n">
+      <c r="M103" s="18" t="n">
         <v>233</v>
       </c>
-      <c r="N103" t="n">
+      <c r="N103" s="18" t="n">
         <v>327</v>
       </c>
-      <c r="O103" t="inlineStr">
+      <c r="O103" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-02.csv</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="19">
-      <c r="A104" s="22" t="n"/>
+      <c r="A104" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>100</v>
+      </c>
+      <c r="C104" t="n">
+        <v>83</v>
+      </c>
+      <c r="D104" t="n">
+        <v>52978</v>
+      </c>
+      <c r="E104" t="n">
+        <v>508034</v>
+      </c>
+      <c r="F104" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="G104" t="n">
+        <v>48</v>
+      </c>
+      <c r="H104" t="n">
+        <v>454</v>
+      </c>
+      <c r="I104" t="n">
+        <v>73</v>
+      </c>
+      <c r="J104" t="n">
+        <v>4089</v>
+      </c>
+      <c r="K104" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="L104" t="n">
+        <v>44</v>
+      </c>
+      <c r="M104" t="n">
+        <v>236</v>
+      </c>
+      <c r="N104" t="n">
+        <v>330</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-03.csv</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="19">
       <c r="A105" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-04
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5795,53 +5795,101 @@
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B104" t="n">
+      <c r="B104" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="C104" t="n">
+      <c r="C104" s="18" t="n">
         <v>83</v>
       </c>
-      <c r="D104" t="n">
+      <c r="D104" s="18" t="n">
         <v>52978</v>
       </c>
-      <c r="E104" t="n">
+      <c r="E104" s="18" t="n">
         <v>508034</v>
       </c>
-      <c r="F104" t="n">
+      <c r="F104" s="18" t="n">
         <v>10.32</v>
       </c>
-      <c r="G104" t="n">
+      <c r="G104" s="18" t="n">
         <v>48</v>
       </c>
-      <c r="H104" t="n">
+      <c r="H104" s="18" t="n">
         <v>454</v>
       </c>
-      <c r="I104" t="n">
+      <c r="I104" s="18" t="n">
         <v>73</v>
       </c>
-      <c r="J104" t="n">
+      <c r="J104" s="18" t="n">
         <v>4089</v>
       </c>
-      <c r="K104" t="n">
+      <c r="K104" s="18" t="n">
         <v>1.79</v>
       </c>
-      <c r="L104" t="n">
+      <c r="L104" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="M104" t="n">
+      <c r="M104" s="18" t="n">
         <v>236</v>
       </c>
-      <c r="N104" t="n">
+      <c r="N104" s="18" t="n">
         <v>330</v>
       </c>
-      <c r="O104" t="inlineStr">
+      <c r="O104" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-03.csv</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="19">
-      <c r="A105" s="22" t="n"/>
+      <c r="A105" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>101</v>
+      </c>
+      <c r="C105" t="n">
+        <v>85</v>
+      </c>
+      <c r="D105" t="n">
+        <v>56369</v>
+      </c>
+      <c r="E105" t="n">
+        <v>613092</v>
+      </c>
+      <c r="F105" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="G105" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="H105" t="n">
+        <v>453</v>
+      </c>
+      <c r="I105" t="n">
+        <v>74</v>
+      </c>
+      <c r="J105" t="n">
+        <v>4106</v>
+      </c>
+      <c r="K105" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L105" t="n">
+        <v>45</v>
+      </c>
+      <c r="M105" t="n">
+        <v>235</v>
+      </c>
+      <c r="N105" t="n">
+        <v>331</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-04.csv</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="19">
       <c r="A106" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-05
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5846,53 +5846,101 @@
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B105" t="n">
+      <c r="B105" s="18" t="n">
         <v>101</v>
       </c>
-      <c r="C105" t="n">
+      <c r="C105" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="D105" t="n">
+      <c r="D105" s="18" t="n">
         <v>56369</v>
       </c>
-      <c r="E105" t="n">
+      <c r="E105" s="18" t="n">
         <v>613092</v>
       </c>
-      <c r="F105" t="n">
+      <c r="F105" s="18" t="n">
         <v>9.1</v>
       </c>
-      <c r="G105" t="n">
+      <c r="G105" s="18" t="n">
         <v>48.6</v>
       </c>
-      <c r="H105" t="n">
+      <c r="H105" s="18" t="n">
         <v>453</v>
       </c>
-      <c r="I105" t="n">
+      <c r="I105" s="18" t="n">
         <v>74</v>
       </c>
-      <c r="J105" t="n">
+      <c r="J105" s="18" t="n">
         <v>4106</v>
       </c>
-      <c r="K105" t="n">
+      <c r="K105" s="18" t="n">
         <v>1.8</v>
       </c>
-      <c r="L105" t="n">
+      <c r="L105" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="M105" t="n">
+      <c r="M105" s="18" t="n">
         <v>235</v>
       </c>
-      <c r="N105" t="n">
+      <c r="N105" s="18" t="n">
         <v>331</v>
       </c>
-      <c r="O105" t="inlineStr">
+      <c r="O105" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-04.csv</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="19">
-      <c r="A106" s="22" t="n"/>
+      <c r="A106" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>106</v>
+      </c>
+      <c r="C106" t="n">
+        <v>86</v>
+      </c>
+      <c r="D106" t="n">
+        <v>58550</v>
+      </c>
+      <c r="E106" t="n">
+        <v>545194</v>
+      </c>
+      <c r="F106" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="G106" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H106" t="n">
+        <v>451</v>
+      </c>
+      <c r="I106" t="n">
+        <v>75</v>
+      </c>
+      <c r="J106" t="n">
+        <v>4116</v>
+      </c>
+      <c r="K106" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="L106" t="n">
+        <v>44</v>
+      </c>
+      <c r="M106" t="n">
+        <v>235</v>
+      </c>
+      <c r="N106" t="n">
+        <v>330</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-05.csv</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="19">
       <c r="A107" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-06
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5897,53 +5897,101 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B106" t="n">
+      <c r="B106" s="18" t="n">
         <v>106</v>
       </c>
-      <c r="C106" t="n">
+      <c r="C106" s="18" t="n">
         <v>86</v>
       </c>
-      <c r="D106" t="n">
+      <c r="D106" s="18" t="n">
         <v>58550</v>
       </c>
-      <c r="E106" t="n">
+      <c r="E106" s="18" t="n">
         <v>545194</v>
       </c>
-      <c r="F106" t="n">
+      <c r="F106" s="18" t="n">
         <v>10.64</v>
       </c>
-      <c r="G106" t="n">
+      <c r="G106" s="18" t="n">
         <v>48.9</v>
       </c>
-      <c r="H106" t="n">
+      <c r="H106" s="18" t="n">
         <v>451</v>
       </c>
-      <c r="I106" t="n">
+      <c r="I106" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="J106" t="n">
+      <c r="J106" s="18" t="n">
         <v>4116</v>
       </c>
-      <c r="K106" t="n">
+      <c r="K106" s="18" t="n">
         <v>1.82</v>
       </c>
-      <c r="L106" t="n">
+      <c r="L106" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="M106" t="n">
+      <c r="M106" s="18" t="n">
         <v>235</v>
       </c>
-      <c r="N106" t="n">
+      <c r="N106" s="18" t="n">
         <v>330</v>
       </c>
-      <c r="O106" t="inlineStr">
+      <c r="O106" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-05.csv</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="19">
-      <c r="A107" s="22" t="n"/>
+      <c r="A107" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>109</v>
+      </c>
+      <c r="C107" t="n">
+        <v>89</v>
+      </c>
+      <c r="D107" t="n">
+        <v>63438</v>
+      </c>
+      <c r="E107" t="n">
+        <v>569425</v>
+      </c>
+      <c r="F107" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G107" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="H107" t="n">
+        <v>452</v>
+      </c>
+      <c r="I107" t="n">
+        <v>76</v>
+      </c>
+      <c r="J107" t="n">
+        <v>4170</v>
+      </c>
+      <c r="K107" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="L107" t="n">
+        <v>45</v>
+      </c>
+      <c r="M107" t="n">
+        <v>236</v>
+      </c>
+      <c r="N107" t="n">
+        <v>330</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-06.csv</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="19">
       <c r="A108" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-07
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5948,53 +5948,101 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B107" t="n">
+      <c r="B107" s="18" t="n">
         <v>109</v>
       </c>
-      <c r="C107" t="n">
+      <c r="C107" s="18" t="n">
         <v>89</v>
       </c>
-      <c r="D107" t="n">
+      <c r="D107" s="18" t="n">
         <v>63438</v>
       </c>
-      <c r="E107" t="n">
+      <c r="E107" s="18" t="n">
         <v>569425</v>
       </c>
-      <c r="F107" t="n">
+      <c r="F107" s="18" t="n">
         <v>11.04</v>
       </c>
-      <c r="G107" t="n">
+      <c r="G107" s="18" t="n">
         <v>49.4</v>
       </c>
-      <c r="H107" t="n">
+      <c r="H107" s="18" t="n">
         <v>452</v>
       </c>
-      <c r="I107" t="n">
+      <c r="I107" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="J107" t="n">
+      <c r="J107" s="18" t="n">
         <v>4170</v>
       </c>
-      <c r="K107" t="n">
+      <c r="K107" s="18" t="n">
         <v>1.82</v>
       </c>
-      <c r="L107" t="n">
+      <c r="L107" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="M107" t="n">
+      <c r="M107" s="18" t="n">
         <v>236</v>
       </c>
-      <c r="N107" t="n">
+      <c r="N107" s="18" t="n">
         <v>330</v>
       </c>
-      <c r="O107" t="inlineStr">
+      <c r="O107" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-06.csv</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="19">
-      <c r="A108" s="22" t="n"/>
+      <c r="A108" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>111</v>
+      </c>
+      <c r="C108" t="n">
+        <v>92</v>
+      </c>
+      <c r="D108" t="n">
+        <v>66840</v>
+      </c>
+      <c r="E108" t="n">
+        <v>583544</v>
+      </c>
+      <c r="F108" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="G108" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="H108" t="n">
+        <v>451</v>
+      </c>
+      <c r="I108" t="n">
+        <v>82</v>
+      </c>
+      <c r="J108" t="n">
+        <v>4219</v>
+      </c>
+      <c r="K108" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="L108" t="n">
+        <v>43</v>
+      </c>
+      <c r="M108" t="n">
+        <v>238</v>
+      </c>
+      <c r="N108" t="n">
+        <v>328</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-07.csv</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="19">
       <c r="A109" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-08
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -5999,53 +5999,101 @@
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B108" t="n">
+      <c r="B108" s="18" t="n">
         <v>111</v>
       </c>
-      <c r="C108" t="n">
+      <c r="C108" s="18" t="n">
         <v>92</v>
       </c>
-      <c r="D108" t="n">
+      <c r="D108" s="18" t="n">
         <v>66840</v>
       </c>
-      <c r="E108" t="n">
+      <c r="E108" s="18" t="n">
         <v>583544</v>
       </c>
-      <c r="F108" t="n">
+      <c r="F108" s="18" t="n">
         <v>11.36</v>
       </c>
-      <c r="G108" t="n">
+      <c r="G108" s="18" t="n">
         <v>50.1</v>
       </c>
-      <c r="H108" t="n">
+      <c r="H108" s="18" t="n">
         <v>451</v>
       </c>
-      <c r="I108" t="n">
+      <c r="I108" s="18" t="n">
         <v>82</v>
       </c>
-      <c r="J108" t="n">
+      <c r="J108" s="18" t="n">
         <v>4219</v>
       </c>
-      <c r="K108" t="n">
+      <c r="K108" s="18" t="n">
         <v>1.94</v>
       </c>
-      <c r="L108" t="n">
+      <c r="L108" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="M108" t="n">
+      <c r="M108" s="18" t="n">
         <v>238</v>
       </c>
-      <c r="N108" t="n">
+      <c r="N108" s="18" t="n">
         <v>328</v>
       </c>
-      <c r="O108" t="inlineStr">
+      <c r="O108" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-07.csv</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="19">
-      <c r="A109" s="22" t="n"/>
+      <c r="A109" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>112</v>
+      </c>
+      <c r="C109" t="n">
+        <v>96</v>
+      </c>
+      <c r="D109" t="n">
+        <v>74482</v>
+      </c>
+      <c r="E109" t="n">
+        <v>622124</v>
+      </c>
+      <c r="F109" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G109" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="H109" t="n">
+        <v>447</v>
+      </c>
+      <c r="I109" t="n">
+        <v>86</v>
+      </c>
+      <c r="J109" t="n">
+        <v>4241</v>
+      </c>
+      <c r="K109" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="L109" t="n">
+        <v>41</v>
+      </c>
+      <c r="M109" t="n">
+        <v>231</v>
+      </c>
+      <c r="N109" t="n">
+        <v>324</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-08.csv</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="19">
       <c r="A110" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-09
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -6050,53 +6050,101 @@
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B109" t="n">
+      <c r="B109" s="18" t="n">
         <v>112</v>
       </c>
-      <c r="C109" t="n">
+      <c r="C109" s="18" t="n">
         <v>96</v>
       </c>
-      <c r="D109" t="n">
+      <c r="D109" s="18" t="n">
         <v>74482</v>
       </c>
-      <c r="E109" t="n">
+      <c r="E109" s="18" t="n">
         <v>622124</v>
       </c>
-      <c r="F109" t="n">
+      <c r="F109" s="18" t="n">
         <v>11.88</v>
       </c>
-      <c r="G109" t="n">
+      <c r="G109" s="18" t="n">
         <v>50.6</v>
       </c>
-      <c r="H109" t="n">
+      <c r="H109" s="18" t="n">
         <v>447</v>
       </c>
-      <c r="I109" t="n">
+      <c r="I109" s="18" t="n">
         <v>86</v>
       </c>
-      <c r="J109" t="n">
+      <c r="J109" s="18" t="n">
         <v>4241</v>
       </c>
-      <c r="K109" t="n">
+      <c r="K109" s="18" t="n">
         <v>2.03</v>
       </c>
-      <c r="L109" t="n">
+      <c r="L109" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="M109" t="n">
+      <c r="M109" s="18" t="n">
         <v>231</v>
       </c>
-      <c r="N109" t="n">
+      <c r="N109" s="18" t="n">
         <v>324</v>
       </c>
-      <c r="O109" t="inlineStr">
+      <c r="O109" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-08.csv</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="19">
-      <c r="A110" s="22" t="n"/>
+      <c r="A110" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>115</v>
+      </c>
+      <c r="C110" t="n">
+        <v>97</v>
+      </c>
+      <c r="D110" t="n">
+        <v>72979</v>
+      </c>
+      <c r="E110" t="n">
+        <v>579438</v>
+      </c>
+      <c r="F110" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G110" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="H110" t="n">
+        <v>445</v>
+      </c>
+      <c r="I110" t="n">
+        <v>85</v>
+      </c>
+      <c r="J110" t="n">
+        <v>4236</v>
+      </c>
+      <c r="K110" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="L110" t="n">
+        <v>40</v>
+      </c>
+      <c r="M110" t="n">
+        <v>230</v>
+      </c>
+      <c r="N110" t="n">
+        <v>325</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-09.csv</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="19">
       <c r="A111" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-10
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -6101,53 +6101,101 @@
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B110" t="n">
+      <c r="B110" s="18" t="n">
         <v>115</v>
       </c>
-      <c r="C110" t="n">
+      <c r="C110" s="18" t="n">
         <v>97</v>
       </c>
-      <c r="D110" t="n">
+      <c r="D110" s="18" t="n">
         <v>72979</v>
       </c>
-      <c r="E110" t="n">
+      <c r="E110" s="18" t="n">
         <v>579438</v>
       </c>
-      <c r="F110" t="n">
+      <c r="F110" s="18" t="n">
         <v>12.5</v>
       </c>
-      <c r="G110" t="n">
+      <c r="G110" s="18" t="n">
         <v>50.5</v>
       </c>
-      <c r="H110" t="n">
+      <c r="H110" s="18" t="n">
         <v>445</v>
       </c>
-      <c r="I110" t="n">
+      <c r="I110" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="J110" t="n">
+      <c r="J110" s="18" t="n">
         <v>4236</v>
       </c>
-      <c r="K110" t="n">
+      <c r="K110" s="18" t="n">
         <v>2.01</v>
       </c>
-      <c r="L110" t="n">
+      <c r="L110" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="M110" t="n">
+      <c r="M110" s="18" t="n">
         <v>230</v>
       </c>
-      <c r="N110" t="n">
+      <c r="N110" s="18" t="n">
         <v>325</v>
       </c>
-      <c r="O110" t="inlineStr">
+      <c r="O110" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-09.csv</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="19">
-      <c r="A111" s="22" t="n"/>
+      <c r="A111" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>117</v>
+      </c>
+      <c r="C111" t="n">
+        <v>99</v>
+      </c>
+      <c r="D111" t="n">
+        <v>73360</v>
+      </c>
+      <c r="E111" t="n">
+        <v>559465</v>
+      </c>
+      <c r="F111" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="G111" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="H111" t="n">
+        <v>443</v>
+      </c>
+      <c r="I111" t="n">
+        <v>86</v>
+      </c>
+      <c r="J111" t="n">
+        <v>4252</v>
+      </c>
+      <c r="K111" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="L111" t="n">
+        <v>41</v>
+      </c>
+      <c r="M111" t="n">
+        <v>234</v>
+      </c>
+      <c r="N111" t="n">
+        <v>328</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-10.csv</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="19">
       <c r="A112" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-11
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -6152,53 +6152,101 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B111" t="n">
+      <c r="B111" s="18" t="n">
         <v>117</v>
       </c>
-      <c r="C111" t="n">
+      <c r="C111" s="18" t="n">
         <v>99</v>
       </c>
-      <c r="D111" t="n">
+      <c r="D111" s="18" t="n">
         <v>73360</v>
       </c>
-      <c r="E111" t="n">
+      <c r="E111" s="18" t="n">
         <v>559465</v>
       </c>
-      <c r="F111" t="n">
+      <c r="F111" s="18" t="n">
         <v>13.01</v>
       </c>
-      <c r="G111" t="n">
+      <c r="G111" s="18" t="n">
         <v>50.9</v>
       </c>
-      <c r="H111" t="n">
+      <c r="H111" s="18" t="n">
         <v>443</v>
       </c>
-      <c r="I111" t="n">
+      <c r="I111" s="18" t="n">
         <v>86</v>
       </c>
-      <c r="J111" t="n">
+      <c r="J111" s="18" t="n">
         <v>4252</v>
       </c>
-      <c r="K111" t="n">
+      <c r="K111" s="18" t="n">
         <v>2.02</v>
       </c>
-      <c r="L111" t="n">
+      <c r="L111" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="M111" t="n">
+      <c r="M111" s="18" t="n">
         <v>234</v>
       </c>
-      <c r="N111" t="n">
+      <c r="N111" s="18" t="n">
         <v>328</v>
       </c>
-      <c r="O111" t="inlineStr">
+      <c r="O111" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-10.csv</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="19">
-      <c r="A112" s="22" t="n"/>
+      <c r="A112" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>120</v>
+      </c>
+      <c r="C112" t="n">
+        <v>102</v>
+      </c>
+      <c r="D112" t="n">
+        <v>77446</v>
+      </c>
+      <c r="E112" t="n">
+        <v>572843</v>
+      </c>
+      <c r="F112" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="G112" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="H112" t="n">
+        <v>439</v>
+      </c>
+      <c r="I112" t="n">
+        <v>85</v>
+      </c>
+      <c r="J112" t="n">
+        <v>4269</v>
+      </c>
+      <c r="K112" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="L112" t="n">
+        <v>41</v>
+      </c>
+      <c r="M112" t="n">
+        <v>235</v>
+      </c>
+      <c r="N112" t="n">
+        <v>322</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-11.csv</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="19">
       <c r="A113" s="22" t="n"/>

</xml_diff>

<commit_message>
chore(stats): daily cloud snapshot 2026-09-12
</commit_message>
<xml_diff>
--- a/data/baselines/daily_stats_log.xlsx
+++ b/data/baselines/daily_stats_log.xlsx
@@ -6203,53 +6203,101 @@
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B112" t="n">
+      <c r="B112" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="C112" t="n">
+      <c r="C112" s="18" t="n">
         <v>102</v>
       </c>
-      <c r="D112" t="n">
+      <c r="D112" s="18" t="n">
         <v>77446</v>
       </c>
-      <c r="E112" t="n">
+      <c r="E112" s="18" t="n">
         <v>572843</v>
       </c>
-      <c r="F112" t="n">
+      <c r="F112" s="18" t="n">
         <v>13.42</v>
       </c>
-      <c r="G112" t="n">
+      <c r="G112" s="18" t="n">
         <v>51.4</v>
       </c>
-      <c r="H112" t="n">
+      <c r="H112" s="18" t="n">
         <v>439</v>
       </c>
-      <c r="I112" t="n">
+      <c r="I112" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="J112" t="n">
+      <c r="J112" s="18" t="n">
         <v>4269</v>
       </c>
-      <c r="K112" t="n">
+      <c r="K112" s="18" t="n">
         <v>1.99</v>
       </c>
-      <c r="L112" t="n">
+      <c r="L112" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="M112" t="n">
+      <c r="M112" s="18" t="n">
         <v>235</v>
       </c>
-      <c r="N112" t="n">
+      <c r="N112" s="18" t="n">
         <v>322</v>
       </c>
-      <c r="O112" t="inlineStr">
+      <c r="O112" s="18" t="inlineStr">
         <is>
           <t>gsc=gsc_queries_2026-09-11.csv</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="19">
-      <c r="A113" s="22" t="n"/>
+      <c r="A113" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>124</v>
+      </c>
+      <c r="C113" t="n">
+        <v>104</v>
+      </c>
+      <c r="D113" t="n">
+        <v>84808</v>
+      </c>
+      <c r="E113" t="n">
+        <v>624568</v>
+      </c>
+      <c r="F113" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="G113" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="H113" t="n">
+        <v>430</v>
+      </c>
+      <c r="I113" t="n">
+        <v>88</v>
+      </c>
+      <c r="J113" t="n">
+        <v>4240</v>
+      </c>
+      <c r="K113" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="L113" t="n">
+        <v>42</v>
+      </c>
+      <c r="M113" t="n">
+        <v>234</v>
+      </c>
+      <c r="N113" t="n">
+        <v>321</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>gsc=gsc_queries_2026-09-12.csv</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="19">
       <c r="A114" s="22" t="n"/>

</xml_diff>